<commit_message>
Template: labor breakdown block + editable charger-run counts
- Intake LABOR BREAKDOWN (rows 58-60): role/phase, days, $/day — all
  yellow; row 1 defaults to the classic crew rate x schedule days so an
  untouched sheet prices exactly as before. LaborBase = the sum;
  Estimate B22 = LaborBase x (1+contingency); Costs Internal D18 shows
  the blended daily rate so its rate x days x contingency chain still
  ties (verified by evaluation: adding a foreman row moves G18 = B22).
- Wire Runs block: the charger rows' Runs cells are now yellow
  overtypeable too (parallel sets on long DCFC runs), matching the app.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/RFC-Template.xlsx
+++ b/templates/RFC-Template.xlsx
@@ -64,17 +64,18 @@
     <definedName name="TrenchFt">Intake!$B$40</definedName>
     <definedName name="LaborDays">Intake!$B$41</definedName>
     <definedName name="WireTotal">Intake!$H$54</definedName>
-    <definedName name="IncHardware">Intake!$B$57</definedName>
-    <definedName name="IncSitePlan">Intake!$B$58</definedName>
-    <definedName name="IncSLD">Intake!$B$59</definedName>
-    <definedName name="IncCpm">Intake!$B$60</definedName>
-    <definedName name="IncPermits">Intake!$B$61</definedName>
-    <definedName name="IncGpr">Intake!$B$62</definedName>
-    <definedName name="HardwareFactor">Intake!$B$65</definedName>
-    <definedName name="RebateAmt">Intake!$B$66</definedName>
-    <definedName name="NetworkFeeMo">Intake!$B$67</definedName>
-    <definedName name="ContractYears">Intake!$B$68</definedName>
-    <definedName name="ServicePlanYr">Intake!$B$69</definedName>
+    <definedName name="LaborBase">Intake!$D$61</definedName>
+    <definedName name="IncHardware">Intake!$B$64</definedName>
+    <definedName name="IncSitePlan">Intake!$B$65</definedName>
+    <definedName name="IncSLD">Intake!$B$66</definedName>
+    <definedName name="IncCpm">Intake!$B$67</definedName>
+    <definedName name="IncPermits">Intake!$B$68</definedName>
+    <definedName name="IncGpr">Intake!$B$69</definedName>
+    <definedName name="HardwareFactor">Intake!$B$72</definedName>
+    <definedName name="RebateAmt">Intake!$B$73</definedName>
+    <definedName name="NetworkFeeMo">Intake!$B$74</definedName>
+    <definedName name="ContractYears">Intake!$B$75</definedName>
+    <definedName name="ServicePlanYr">Intake!$B$76</definedName>
     <definedName name="SgSuggested">Panel!$F$15</definedName>
     <definedName name="TxKvaConnected">Panel!$F$33</definedName>
     <definedName name="TxKvaSuggested">Panel!$F$35</definedName>
@@ -94,7 +95,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="669" uniqueCount="379">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="678" uniqueCount="388">
   <si>
     <t>RFC INTAKE — EV Charging Project</t>
   </si>
@@ -264,6 +265,27 @@
     <t>Wire total</t>
   </si>
   <si>
+    <t>LABOR BREAKDOWN — add roles/phases; the total feeds the estimate</t>
+  </si>
+  <si>
+    <t>Role / phase</t>
+  </si>
+  <si>
+    <t>Days</t>
+  </si>
+  <si>
+    <t>$ / day</t>
+  </si>
+  <si>
+    <t>Labor $</t>
+  </si>
+  <si>
+    <t>Electrical crew</t>
+  </si>
+  <si>
+    <t>Labor total (before contingency)</t>
+  </si>
+  <si>
     <t>INCLUDED SERVICES (Yes / No)</t>
   </si>
   <si>
@@ -585,7 +607,7 @@
     <t>Construction total (loaded)</t>
   </si>
   <si>
-    <t>Labor (days × rate, contingency-loaded)</t>
+    <t>Labor (breakdown total, contingency-loaded)</t>
   </si>
   <si>
     <t>Sales tax on construction</t>
@@ -1170,10 +1192,16 @@
     <t xml:space="preserve">   labor days, services, commercial terms. Totals show at the bottom of the Intake.</t>
   </si>
   <si>
-    <t>2. WIRE RUNS &amp; FEEDERS: every run's wire size, material (Cu/Al) and one-way ft is editable — like the V18 workbooks. Defaults</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   auto-fill from the model and site distances; overtyping a yellow cell replaces its default formula (re-enter it to restore).</t>
+    <t>2. WIRE RUNS &amp; FEEDERS: every run's wire size, material (Cu/Al), runs and one-way ft is editable — like the V18 workbooks.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Defaults auto-fill from the model and site distances; overtyping a yellow cell replaces its default formula. On long DCFC or</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   feeder runs, extra parallel runs split the amps so each set can use smaller wire — often cheaper than one fat conductor.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   LABOR BREAKDOWN: itemize by role/phase (foreman, crew, flagger…); the total feeds the estimate, contingency-loaded.</t>
   </si>
   <si>
     <t>3. Every price lives on the RateCard (yellow) — hardware, install allowance, gear catalog, wire $/ft (incl. 450 kcmil Cu &amp; Al),</t>
@@ -1464,8 +1492,8 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1896,7 +1924,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H74"/>
+  <dimension ref="A1:H81"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -2285,7 +2313,7 @@
       <c r="C45" s="5">
         <f>IFERROR(VLOOKUP($A$23,ModelTable,15,FALSE),"Cu")</f>
       </c>
-      <c r="D45">
+      <c r="D45" s="5">
         <f>IFERROR($B$23*VLOOKUP($A$23,ModelTable,12,FALSE),0)</f>
       </c>
       <c r="E45">
@@ -2311,7 +2339,7 @@
       <c r="C46" s="5">
         <f>IFERROR(VLOOKUP($A$24,ModelTable,15,FALSE),"Cu")</f>
       </c>
-      <c r="D46">
+      <c r="D46" s="5">
         <f>IFERROR($B$24*VLOOKUP($A$24,ModelTable,12,FALSE),0)</f>
       </c>
       <c r="E46">
@@ -2337,7 +2365,7 @@
       <c r="C47" s="5">
         <f>IFERROR(VLOOKUP($A$25,ModelTable,15,FALSE),"Cu")</f>
       </c>
-      <c r="D47">
+      <c r="D47" s="5">
         <f>IFERROR($B$25*VLOOKUP($A$25,ModelTable,12,FALSE),0)</f>
       </c>
       <c r="E47">
@@ -2363,7 +2391,7 @@
       <c r="C48" s="5">
         <f>IFERROR(VLOOKUP($A$26,ModelTable,15,FALSE),"Cu")</f>
       </c>
-      <c r="D48">
+      <c r="D48" s="5">
         <f>IFERROR($B$26*VLOOKUP($A$26,ModelTable,12,FALSE),0)</f>
       </c>
       <c r="E48">
@@ -2389,7 +2417,7 @@
       <c r="C49" s="5">
         <f>IFERROR(VLOOKUP($A$27,ModelTable,15,FALSE),"Cu")</f>
       </c>
-      <c r="D49">
+      <c r="D49" s="5">
         <f>IFERROR($B$27*VLOOKUP($A$27,ModelTable,12,FALSE),0)</f>
       </c>
       <c r="E49">
@@ -2415,7 +2443,7 @@
       <c r="C50" s="5">
         <f>IFERROR(VLOOKUP($A$28,ModelTable,15,FALSE),"Cu")</f>
       </c>
-      <c r="D50">
+      <c r="D50" s="5">
         <f>IFERROR($B$28*VLOOKUP($A$28,ModelTable,12,FALSE),0)</f>
       </c>
       <c r="E50">
@@ -2522,131 +2550,196 @@
         <v>56</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A57" s="4" t="s">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="B57" s="5" t="s">
+      <c r="B57" s="7" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A58" s="4" t="s">
+      <c r="C57" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="B58" s="5" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A59" s="4" t="s">
+      <c r="D57" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="B59" s="5" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A60" s="4" t="s">
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="B60" s="5" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A61" s="4" t="s">
+      <c r="B58" s="5">
+        <f>LaborDays</f>
+      </c>
+      <c r="C58" s="11">
+        <f>LaborDayRate</f>
+      </c>
+      <c r="D58" s="9">
+        <f>$B$58*$C$58</f>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" s="5"/>
+      <c r="B59" s="5">
+        <v>0</v>
+      </c>
+      <c r="C59" s="11">
+        <v>0</v>
+      </c>
+      <c r="D59" s="9">
+        <f>$B$59*$C$59</f>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60" s="5"/>
+      <c r="B60" s="5">
+        <v>0</v>
+      </c>
+      <c r="C60" s="11">
+        <v>0</v>
+      </c>
+      <c r="D60" s="9">
+        <f>$B$60*$C$60</f>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="B61" s="5" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A62" s="4" t="s">
+      <c r="D61" s="10">
+        <f>SUM(D58:D60)</f>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A63" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="B62" s="5" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A64" s="3" t="s">
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A64" s="4" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B64" s="5" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B65" s="5" t="s">
         <v>65</v>
-      </c>
-      <c r="B65" s="5">
-        <v>1</v>
-      </c>
-      <c r="C65" s="11" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="B66" s="12">
-        <v>0</v>
+      <c r="B66" s="5" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B67" s="12">
-        <v>39.99</v>
+      <c r="B67" s="5" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="B68" s="5">
-        <v>5</v>
+      <c r="B68" s="5" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="B69" s="12">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B69" s="5" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A71" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="B71">
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A72" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B72" s="5">
+        <v>1</v>
+      </c>
+      <c r="C72" s="12" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A73" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="B73" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A74" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="B74" s="11">
+        <v>39.99</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A75" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B75" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A76" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="B76" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A78" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B78">
         <f>AdaVan&amp;" van + "&amp;AdaStd&amp;" standard + "&amp;AdaAmb&amp;" ambulatory"</f>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A72" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B72">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A79" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="B79">
         <f>IF(NDcfc&gt;0,SgSuggested&amp;"A switchgear @ 480V","208V service")&amp;IF(TxKvaSuggested&gt;0," + "&amp;TxKvaSuggested&amp;" kVA step-down TX","")</f>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A73" s="13" t="s">
-        <v>73</v>
-      </c>
-      <c r="B73" s="14">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A80" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="B80" s="14">
         <f>TotalCost</f>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A74" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="B74" s="10">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A81" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B81" s="10">
         <f>CustomerTotal</f>
       </c>
     </row>
@@ -2661,7 +2754,7 @@
     <dataValidation type="list" allowBlank="1" sqref="B45:B53">
       <formula1>RateCard!$A$129:$A$153</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="B57:B62">
+    <dataValidation type="list" sqref="B64:B69">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="C45:C53">
@@ -2675,7 +2768,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A28"/>
+  <dimension ref="A1:A30"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="114" customWidth="1"/>
@@ -2683,142 +2776,152 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>354</v>
+        <v>361</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="63" t="s">
-        <v>355</v>
+        <v>362</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="63" t="s">
-        <v>356</v>
+        <v>363</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="63" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="63" t="s">
-        <v>358</v>
+        <v>365</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="63" t="s">
-        <v>359</v>
+        <v>366</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="63" t="s">
-        <v>360</v>
+        <v>367</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="63" t="s">
-        <v>361</v>
+        <v>368</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="63" t="s">
-        <v>362</v>
+        <v>369</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="63" t="s">
-        <v>363</v>
+        <v>370</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="63" t="s">
-        <v>238</v>
+        <v>371</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" s="16" t="s">
-        <v>364</v>
+      <c r="A12" s="63" t="s">
+        <v>372</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="63" t="s">
-        <v>365</v>
+        <v>245</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" s="63" t="s">
-        <v>366</v>
+      <c r="A14" s="16" t="s">
+        <v>373</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" s="63" t="s">
-        <v>367</v>
+        <v>374</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" s="63" t="s">
-        <v>238</v>
+        <v>375</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" s="16" t="s">
-        <v>368</v>
+      <c r="A17" s="63" t="s">
+        <v>376</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="63" t="s">
-        <v>369</v>
+        <v>245</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" s="63" t="s">
-        <v>370</v>
+      <c r="A19" s="16" t="s">
+        <v>377</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" s="63" t="s">
-        <v>238</v>
+        <v>378</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" s="16" t="s">
-        <v>371</v>
+      <c r="A21" s="63" t="s">
+        <v>379</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" s="63" t="s">
-        <v>372</v>
+        <v>245</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" s="63" t="s">
-        <v>373</v>
+      <c r="A23" s="16" t="s">
+        <v>380</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="63" t="s">
-        <v>374</v>
+        <v>381</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" s="63" t="s">
-        <v>375</v>
+        <v>382</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" s="63" t="s">
-        <v>376</v>
+        <v>383</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" s="63" t="s">
-        <v>377</v>
+        <v>384</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" s="63" t="s">
-        <v>378</v>
+        <v>385</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" s="63" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" s="63" t="s">
+        <v>387</v>
       </c>
     </row>
   </sheetData>
@@ -2839,12 +2942,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="15" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -2855,16 +2958,16 @@
         <v>19</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -2989,7 +3092,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="F11">
         <f>SUM(F5:F10)</f>
@@ -2997,7 +3100,7 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="F12">
         <f>IF(AND(NDcfc&gt;0,NumL2&gt;0),TxKvaConnected*1000/(480*SQRT(3)),0)</f>
@@ -3005,7 +3108,7 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="F13">
         <f>F11+F12</f>
@@ -3013,7 +3116,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="F14">
         <f>F13*1.25</f>
@@ -3021,7 +3124,7 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="F15">
         <f>IF(NDcfc&gt;0,INDEX(SgSizes,MIN(ROWS(SgSizes),COUNTIF(SgSizes,"&lt;"&amp;F14)+1)),0)</f>
@@ -3029,7 +3132,7 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="F16" s="9">
         <f>IF(NDcfc&gt;0,VLOOKUP(SgSuggested,SgTable,2,FALSE),0)</f>
@@ -3037,7 +3140,7 @@
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -3048,16 +3151,16 @@
         <v>19</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
@@ -3182,7 +3285,7 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="F26">
         <f>SUM(F20:F25)</f>
@@ -3190,7 +3293,7 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="F27">
         <f>F26*1.25</f>
@@ -3198,7 +3301,7 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="F28">
         <f>IF(NumL2&gt;0,INDEX(PnlSizes,MIN(ROWS(PnlSizes),COUNTIF(PnlSizes,"&lt;"&amp;F27)+1)),0)</f>
@@ -3206,7 +3309,7 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="F29">
         <f>IF(NumL2=0,"—",IF(F28&gt;=1000,"Distribution panel","Sub-panel"))</f>
@@ -3214,7 +3317,7 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="F30" s="9">
         <f>IF(NumL2&gt;0,VLOOKUP(F28,PnlTable,2,FALSE),0)</f>
@@ -3222,12 +3325,12 @@
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="4" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="F33">
         <f>IF(AND(NDcfc&gt;0,NumL2&gt;0),F26*208*SQRT(3)/1000,0)</f>
@@ -3235,7 +3338,7 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="F34">
         <f>F33*1.25</f>
@@ -3243,7 +3346,7 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="F35">
         <f>IF(F33&gt;0,INDEX(TxSizes,MIN(ROWS(TxSizes),COUNTIF(TxSizes,"&lt;"&amp;F34)+1)),0)</f>
@@ -3251,7 +3354,7 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="F36" s="9">
         <f>IF(F35&gt;0,VLOOKUP(F35,TxTable,2,FALSE),0)</f>
@@ -3259,7 +3362,7 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="4" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="F37">
         <f>IF(F35&gt;0,F35*1000/(480*SQRT(3)),0)</f>
@@ -3267,7 +3370,7 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="F38">
         <f>IF(F35&gt;0,INDEX(StdBrk,MIN(ROWS(StdBrk),COUNTIF(StdBrk,"&lt;"&amp;F37*1.25)+1)),0)</f>
@@ -3275,7 +3378,7 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="4" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="F39" s="9">
         <f>IF(F38&gt;0,IFERROR(VLOOKUP(F38,BrkTbl480,2,FALSE),0),0)</f>
@@ -3283,7 +3386,7 @@
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
@@ -3291,19 +3394,19 @@
         <v>18</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="D42" s="7" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="E42" s="7" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="F42" s="7" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
@@ -3428,7 +3531,7 @@
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="F49" s="9">
         <f>SUM(F43:F48)+F39</f>
@@ -3436,7 +3539,7 @@
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="16" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="F51" s="17">
         <f>F16+F30+F36+F49</f>
@@ -3444,7 +3547,7 @@
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" s="18" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
     </row>
   </sheetData>
@@ -3481,7 +3584,7 @@
   <sheetData>
     <row r="1" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B1" s="19" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="C1" s="19"/>
       <c r="D1" s="19"/>
@@ -3499,30 +3602,30 @@
     </row>
     <row r="2" spans="18:18" x14ac:dyDescent="0.25">
       <c r="R2" s="20" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
     </row>
     <row r="3" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B3" s="21" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="C3" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="D3" s="21" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="E3" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="H3" s="21" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="I3" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="M3" s="21" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="N3">
         <f>SgSuggested&amp;" A 3P"</f>
@@ -3536,19 +3639,19 @@
     </row>
     <row r="4" spans="4:20" x14ac:dyDescent="0.25">
       <c r="D4" s="21" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="E4">
         <f>"UTILITY"</f>
       </c>
       <c r="H4" s="21" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="I4" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="M4" s="21" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="N4">
         <f>SgSuggested&amp;" A"</f>
@@ -3562,22 +3665,22 @@
     </row>
     <row r="5" spans="4:20" x14ac:dyDescent="0.25">
       <c r="D5" s="21" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="E5" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="H5" s="21" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="I5" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="M5" s="21" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="N5" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="S5">
         <f>IF(Intake!$D$25="DCFC",Intake!$B$25*IFERROR(VLOOKUP(Intake!$A$25,ModelTable,7,FALSE),0),0)</f>
@@ -3596,40 +3699,40 @@
     </row>
     <row r="7" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B7" s="22" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="C7" s="22" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="D7" s="22" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="E7" s="22" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="F7" s="22" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="G7" s="22"/>
       <c r="H7" s="22" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="I7" s="22"/>
       <c r="J7" s="22" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="K7" s="22"/>
       <c r="L7" s="22" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="M7" s="22" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="N7" s="22" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="O7" s="22" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="S7">
         <f>IF(Intake!$D$27="DCFC",Intake!$B$27*IFERROR(VLOOKUP(Intake!$A$27,ModelTable,7,FALSE),0),0)</f>
@@ -3640,7 +3743,7 @@
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="B8" s="23">
         <v>1</v>
@@ -3677,7 +3780,7 @@
         <v>2</v>
       </c>
       <c r="P8" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="S8">
         <f>IF(Intake!$D$28="DCFC",Intake!$B$28*IFERROR(VLOOKUP(Intake!$A$28,ModelTable,7,FALSE),0),0)</f>
@@ -3688,7 +3791,7 @@
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="B9" s="23">
         <v>3</v>
@@ -3717,10 +3820,10 @@
         <v>4</v>
       </c>
       <c r="P9" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="R9" s="24" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="S9">
         <f>SUM(S3:S8)</f>
@@ -3728,7 +3831,7 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="B10" s="23">
         <v>5</v>
@@ -3757,12 +3860,12 @@
         <v>6</v>
       </c>
       <c r="P10" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="B11" s="23">
         <v>7</v>
@@ -3799,12 +3902,12 @@
         <v>8</v>
       </c>
       <c r="P11" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="B12" s="23">
         <v>9</v>
@@ -3833,7 +3936,7 @@
         <v>10</v>
       </c>
       <c r="P12" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="S12">
         <v>1</v>
@@ -3865,7 +3968,7 @@
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="B13" s="23">
         <v>11</v>
@@ -3894,7 +3997,7 @@
         <v>12</v>
       </c>
       <c r="P13" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="S13">
         <v>2</v>
@@ -3926,7 +4029,7 @@
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="B14" s="23">
         <v>13</v>
@@ -3963,7 +4066,7 @@
         <v>14</v>
       </c>
       <c r="P14" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="S14">
         <v>3</v>
@@ -3995,7 +4098,7 @@
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="B15" s="23">
         <v>15</v>
@@ -4024,7 +4127,7 @@
         <v>16</v>
       </c>
       <c r="P15" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="S15">
         <v>4</v>
@@ -4056,7 +4159,7 @@
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="B16" s="23">
         <v>17</v>
@@ -4085,7 +4188,7 @@
         <v>18</v>
       </c>
       <c r="P16" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="S16">
         <v>5</v>
@@ -4117,7 +4220,7 @@
     </row>
     <row r="17" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="B17" s="23">
         <v>19</v>
@@ -4154,7 +4257,7 @@
         <v>20</v>
       </c>
       <c r="P17" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="S17">
         <v>6</v>
@@ -4186,7 +4289,7 @@
     </row>
     <row r="18" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="B18" s="23">
         <v>21</v>
@@ -4215,7 +4318,7 @@
         <v>22</v>
       </c>
       <c r="P18" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="S18">
         <v>7</v>
@@ -4247,7 +4350,7 @@
     </row>
     <row r="19" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="B19" s="23">
         <v>23</v>
@@ -4276,7 +4379,7 @@
         <v>24</v>
       </c>
       <c r="P19" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="S19">
         <v>8</v>
@@ -4308,7 +4411,7 @@
     </row>
     <row r="20" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="B20" s="23">
         <v>25</v>
@@ -4345,7 +4448,7 @@
         <v>26</v>
       </c>
       <c r="P20" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="S20">
         <v>9</v>
@@ -4377,7 +4480,7 @@
     </row>
     <row r="21" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="B21" s="23">
         <v>27</v>
@@ -4406,7 +4509,7 @@
         <v>28</v>
       </c>
       <c r="P21" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="S21">
         <v>10</v>
@@ -4438,7 +4541,7 @@
     </row>
     <row r="22" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="B22" s="23">
         <v>29</v>
@@ -4467,7 +4570,7 @@
         <v>30</v>
       </c>
       <c r="P22" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="S22">
         <v>11</v>
@@ -4499,7 +4602,7 @@
     </row>
     <row r="23" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="B23" s="23">
         <v>31</v>
@@ -4536,7 +4639,7 @@
         <v>32</v>
       </c>
       <c r="P23" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="S23">
         <v>12</v>
@@ -4568,7 +4671,7 @@
     </row>
     <row r="24" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="B24" s="23">
         <v>33</v>
@@ -4597,7 +4700,7 @@
         <v>34</v>
       </c>
       <c r="P24" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="S24">
         <v>13</v>
@@ -4629,7 +4732,7 @@
     </row>
     <row r="25" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="B25" s="23">
         <v>35</v>
@@ -4658,7 +4761,7 @@
         <v>36</v>
       </c>
       <c r="P25" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="S25">
         <v>14</v>
@@ -4690,7 +4793,7 @@
     </row>
     <row r="26" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="B26" s="23">
         <v>37</v>
@@ -4727,7 +4830,7 @@
         <v>38</v>
       </c>
       <c r="P26" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="S26">
         <v>15</v>
@@ -4759,7 +4862,7 @@
     </row>
     <row r="27" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="B27" s="23">
         <v>39</v>
@@ -4788,7 +4891,7 @@
         <v>40</v>
       </c>
       <c r="P27" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="S27">
         <v>16</v>
@@ -4820,7 +4923,7 @@
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="B28" s="23">
         <v>41</v>
@@ -4849,12 +4952,12 @@
         <v>42</v>
       </c>
       <c r="P28" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
     </row>
     <row r="29" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="B29" s="23">
         <v>43</v>
@@ -4891,12 +4994,12 @@
         <v>44</v>
       </c>
       <c r="P29" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="B30" s="23">
         <v>45</v>
@@ -4925,12 +5028,12 @@
         <v>46</v>
       </c>
       <c r="P30" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="B31" s="23">
         <v>47</v>
@@ -4959,12 +5062,12 @@
         <v>48</v>
       </c>
       <c r="P31" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
     </row>
     <row r="33" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C33" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="F33" s="25">
         <f>SUM(F8:G31)</f>
@@ -4979,7 +5082,7 @@
       </c>
       <c r="K33" s="25"/>
       <c r="L33" s="21" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="M33" s="21"/>
       <c r="N33" s="25">
@@ -4988,7 +5091,7 @@
     </row>
     <row r="34" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C34" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="F34" s="25">
         <f>F33*1.25</f>
@@ -5003,7 +5106,7 @@
       </c>
       <c r="K34" s="25"/>
       <c r="L34" s="21" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="M34" s="21"/>
       <c r="N34" s="25">
@@ -5012,7 +5115,7 @@
     </row>
     <row r="35" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C35" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="F35" s="25">
         <f>MAX($F$34,$H$34,$J$34)</f>
@@ -5027,7 +5130,7 @@
       </c>
       <c r="K35" s="25"/>
       <c r="L35" s="21" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="M35" s="21"/>
       <c r="N35" s="26">
@@ -5036,7 +5139,7 @@
     </row>
     <row r="36" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C36" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="F36" s="26">
         <f>F35/(480/SQRT(3))</f>
@@ -5051,7 +5154,7 @@
       </c>
       <c r="K36" s="26"/>
       <c r="L36" s="21" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="M36" s="21"/>
       <c r="N36">
@@ -5119,7 +5222,7 @@
   <sheetData>
     <row r="1" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B1" s="19" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="C1" s="19"/>
       <c r="D1" s="19"/>
@@ -5137,30 +5240,30 @@
     </row>
     <row r="2" spans="18:18" x14ac:dyDescent="0.25">
       <c r="R2" s="20" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
     </row>
     <row r="3" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B3" s="21" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="C3" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="D3" s="21" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="E3" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="H3" s="21" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="I3" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="M3" s="21" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="N3">
         <f>Panel!$F$28&amp;" A 3P"</f>
@@ -5174,19 +5277,19 @@
     </row>
     <row r="4" spans="4:20" x14ac:dyDescent="0.25">
       <c r="D4" s="21" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="E4">
         <f>IF(TxKvaSuggested&gt;0,"EV_MAIN VIA "&amp;TxKvaSuggested&amp;" KVA XFMR","UTILITY")</f>
       </c>
       <c r="H4" s="21" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="I4" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="M4" s="21" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="N4">
         <f>Panel!$F$28&amp;" A"</f>
@@ -5200,22 +5303,22 @@
     </row>
     <row r="5" spans="4:20" x14ac:dyDescent="0.25">
       <c r="D5" s="21" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="E5" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="H5" s="21" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="I5" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="M5" s="21" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="N5" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="S5">
         <f>IF(Intake!$D$25="L2",Intake!$B$25*IFERROR(VLOOKUP(Intake!$A$25,ModelTable,7,FALSE),0),0)</f>
@@ -5234,40 +5337,40 @@
     </row>
     <row r="7" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B7" s="22" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="C7" s="22" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="D7" s="22" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="E7" s="22" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="F7" s="22" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="G7" s="22"/>
       <c r="H7" s="22" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="I7" s="22"/>
       <c r="J7" s="22" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="K7" s="22"/>
       <c r="L7" s="22" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="M7" s="22" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="N7" s="22" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="O7" s="22" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="S7">
         <f>IF(Intake!$D$27="L2",Intake!$B$27*IFERROR(VLOOKUP(Intake!$A$27,ModelTable,7,FALSE),0),0)</f>
@@ -5278,7 +5381,7 @@
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="B8" s="23">
         <v>1</v>
@@ -5315,7 +5418,7 @@
         <v>2</v>
       </c>
       <c r="P8" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="S8">
         <f>IF(Intake!$D$28="L2",Intake!$B$28*IFERROR(VLOOKUP(Intake!$A$28,ModelTable,7,FALSE),0),0)</f>
@@ -5326,7 +5429,7 @@
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="B9" s="23">
         <v>3</v>
@@ -5355,10 +5458,10 @@
         <v>4</v>
       </c>
       <c r="P9" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="R9" s="24" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="S9">
         <f>SUM(S3:S8)</f>
@@ -5366,7 +5469,7 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="B10" s="23">
         <v>5</v>
@@ -5403,12 +5506,12 @@
         <v>6</v>
       </c>
       <c r="P10" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="B11" s="23">
         <v>7</v>
@@ -5437,12 +5540,12 @@
         <v>8</v>
       </c>
       <c r="P11" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="B12" s="23">
         <v>9</v>
@@ -5479,7 +5582,7 @@
         <v>10</v>
       </c>
       <c r="P12" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="S12">
         <v>1</v>
@@ -5511,7 +5614,7 @@
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="B13" s="23">
         <v>11</v>
@@ -5540,7 +5643,7 @@
         <v>12</v>
       </c>
       <c r="P13" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="S13">
         <v>2</v>
@@ -5572,7 +5675,7 @@
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="B14" s="23">
         <v>13</v>
@@ -5609,7 +5712,7 @@
         <v>14</v>
       </c>
       <c r="P14" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="S14">
         <v>3</v>
@@ -5641,7 +5744,7 @@
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="B15" s="23">
         <v>15</v>
@@ -5670,7 +5773,7 @@
         <v>16</v>
       </c>
       <c r="P15" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="S15">
         <v>4</v>
@@ -5702,7 +5805,7 @@
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="B16" s="23">
         <v>17</v>
@@ -5739,7 +5842,7 @@
         <v>18</v>
       </c>
       <c r="P16" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="S16">
         <v>5</v>
@@ -5771,7 +5874,7 @@
     </row>
     <row r="17" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="B17" s="23">
         <v>19</v>
@@ -5800,7 +5903,7 @@
         <v>20</v>
       </c>
       <c r="P17" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="S17">
         <v>6</v>
@@ -5832,7 +5935,7 @@
     </row>
     <row r="18" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="B18" s="23">
         <v>21</v>
@@ -5869,7 +5972,7 @@
         <v>22</v>
       </c>
       <c r="P18" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="S18">
         <v>7</v>
@@ -5901,7 +6004,7 @@
     </row>
     <row r="19" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="B19" s="23">
         <v>23</v>
@@ -5930,7 +6033,7 @@
         <v>24</v>
       </c>
       <c r="P19" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="S19">
         <v>8</v>
@@ -5962,7 +6065,7 @@
     </row>
     <row r="20" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="B20" s="23">
         <v>25</v>
@@ -5999,7 +6102,7 @@
         <v>26</v>
       </c>
       <c r="P20" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="S20">
         <v>9</v>
@@ -6031,7 +6134,7 @@
     </row>
     <row r="21" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="B21" s="23">
         <v>27</v>
@@ -6060,7 +6163,7 @@
         <v>28</v>
       </c>
       <c r="P21" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="S21">
         <v>10</v>
@@ -6092,7 +6195,7 @@
     </row>
     <row r="22" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="B22" s="23">
         <v>29</v>
@@ -6129,7 +6232,7 @@
         <v>30</v>
       </c>
       <c r="P22" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="S22">
         <v>11</v>
@@ -6161,7 +6264,7 @@
     </row>
     <row r="23" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="B23" s="23">
         <v>31</v>
@@ -6190,7 +6293,7 @@
         <v>32</v>
       </c>
       <c r="P23" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="S23">
         <v>12</v>
@@ -6222,7 +6325,7 @@
     </row>
     <row r="24" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="B24" s="23">
         <v>33</v>
@@ -6259,7 +6362,7 @@
         <v>34</v>
       </c>
       <c r="P24" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="S24">
         <v>13</v>
@@ -6291,7 +6394,7 @@
     </row>
     <row r="25" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="B25" s="23">
         <v>35</v>
@@ -6320,7 +6423,7 @@
         <v>36</v>
       </c>
       <c r="P25" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="S25">
         <v>14</v>
@@ -6352,7 +6455,7 @@
     </row>
     <row r="26" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="B26" s="23">
         <v>37</v>
@@ -6389,7 +6492,7 @@
         <v>38</v>
       </c>
       <c r="P26" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="S26">
         <v>15</v>
@@ -6421,7 +6524,7 @@
     </row>
     <row r="27" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="B27" s="23">
         <v>39</v>
@@ -6450,7 +6553,7 @@
         <v>40</v>
       </c>
       <c r="P27" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="S27">
         <v>16</v>
@@ -6482,7 +6585,7 @@
     </row>
     <row r="28" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="B28" s="23">
         <v>41</v>
@@ -6519,7 +6622,7 @@
         <v>42</v>
       </c>
       <c r="P28" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="S28">
         <v>17</v>
@@ -6551,7 +6654,7 @@
     </row>
     <row r="29" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="B29" s="23">
         <v>43</v>
@@ -6580,7 +6683,7 @@
         <v>44</v>
       </c>
       <c r="P29" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="S29">
         <v>18</v>
@@ -6612,7 +6715,7 @@
     </row>
     <row r="30" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="B30" s="23">
         <v>45</v>
@@ -6649,7 +6752,7 @@
         <v>46</v>
       </c>
       <c r="P30" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="S30">
         <v>19</v>
@@ -6681,7 +6784,7 @@
     </row>
     <row r="31" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="B31" s="23">
         <v>47</v>
@@ -6710,7 +6813,7 @@
         <v>48</v>
       </c>
       <c r="P31" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="S31">
         <v>20</v>
@@ -6771,7 +6874,7 @@
     </row>
     <row r="33" spans="3:27" x14ac:dyDescent="0.25">
       <c r="C33" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="F33" s="25">
         <f>SUM(F8:G31)</f>
@@ -6786,7 +6889,7 @@
       </c>
       <c r="K33" s="25"/>
       <c r="L33" s="21" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="M33" s="21"/>
       <c r="N33" s="25">
@@ -6822,7 +6925,7 @@
     </row>
     <row r="34" spans="3:27" x14ac:dyDescent="0.25">
       <c r="C34" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="F34" s="25">
         <f>F33*1.25</f>
@@ -6837,7 +6940,7 @@
       </c>
       <c r="K34" s="25"/>
       <c r="L34" s="21" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="M34" s="21"/>
       <c r="N34" s="25">
@@ -6873,7 +6976,7 @@
     </row>
     <row r="35" spans="3:27" x14ac:dyDescent="0.25">
       <c r="C35" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="F35" s="25">
         <f>MAX($F$34,$H$34,$J$34)</f>
@@ -6888,7 +6991,7 @@
       </c>
       <c r="K35" s="25"/>
       <c r="L35" s="21" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="M35" s="21"/>
       <c r="N35" s="26">
@@ -6924,7 +7027,7 @@
     </row>
     <row r="36" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C36" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="F36" s="26">
         <f>F35/120</f>
@@ -6939,7 +7042,7 @@
       </c>
       <c r="K36" s="26"/>
       <c r="L36" s="21" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="M36" s="21"/>
       <c r="N36">
@@ -6991,17 +7094,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="15" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="B4">
         <f>LaborDays</f>
@@ -7009,13 +7112,13 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="28" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="B6" s="29"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="B7" s="9">
         <f>WireTotal+SUM(Intake!E23:E28)</f>
@@ -7023,7 +7126,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="B8" s="9">
         <f>GearTotal</f>
@@ -7031,7 +7134,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="B9" s="9">
         <f>TrenchFt*TrenchRate*VLOOKUP(Terrain,TerrainTable,2,FALSE)</f>
@@ -7039,7 +7142,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="B10" s="9">
         <f>IF(NTotal&gt;0,CivilBase,0)+NDcfc*CivilDcfc+NumL2*CivilL2</f>
@@ -7047,7 +7150,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="B11" s="9">
         <f>NDcfc*SignageDcfc+NumL2*SignageL2</f>
@@ -7055,7 +7158,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="B12" s="9">
         <f>AdaCost</f>
@@ -7063,7 +7166,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="B13" s="9">
         <f>TrenchFt*VLOOKUP(Terrain,TerrainTable,5,FALSE)</f>
@@ -7071,7 +7174,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="B14" s="9">
         <f>IF(IncGpr="Yes",MAX(1,ROUNDUP(TrenchFt/GprFtPerDay,0))*GprDayRate,0)</f>
@@ -7079,7 +7182,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="B15" s="9">
         <f>IF(NTotal&gt;0,EquipBase+EquipPerDay*LaborDays,0)</f>
@@ -7087,7 +7190,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="B16" s="9">
         <f>IF(IncPermits="Yes",200+60*NTotal,0)</f>
@@ -7095,7 +7198,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="B17" s="9">
         <f>IF(IncPermits="Yes",IF(NDcfc&gt;0,2500+TransformerPad,800),0)</f>
@@ -7103,7 +7206,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="B18" s="9">
         <f>SUM(B7:B17)</f>
@@ -7111,7 +7214,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="B19" s="9">
         <f>B18*ContingencyPct</f>
@@ -7119,7 +7222,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="B20" s="10">
         <f>B18+B19</f>
@@ -7127,15 +7230,15 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="B22" s="9">
-        <f>LaborDays*LaborDayRate*(1+ContingencyPct)</f>
+        <f>LaborBase*(1+ContingencyPct)</f>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="B23" s="9">
         <f>ConstructionTotal*TaxPct</f>
@@ -7143,7 +7246,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="30" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="B24" s="9">
         <f>ConstructionTotal+LaborCost</f>
@@ -7151,13 +7254,13 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="28" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="B26" s="29"/>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>167</v>
+        <v>174</v>
       </c>
       <c r="B27" s="9">
         <f>IF(IncHardware="Yes",SUM(Intake!F23:F28)*HardwareFactor,0)</f>
@@ -7165,7 +7268,7 @@
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="B28" s="9">
         <f>IF(IncHardware="Yes",CommDcfc*NDcfc+CommL2*NumL2,0)</f>
@@ -7173,7 +7276,7 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="B29" s="9">
         <f>IF(IncHardware="Yes",NPorts*NetworkFeeMo*12*ContractYears,0)</f>
@@ -7181,7 +7284,7 @@
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="B30" s="9">
         <f>IF(IncHardware="Yes",ServicePlanYr*ContractYears,0)</f>
@@ -7189,7 +7292,7 @@
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="B31" s="9">
         <f>B27*TaxPct</f>
@@ -7197,13 +7300,13 @@
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="28" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="B33" s="29"/>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="B34" s="9">
         <f>IF(IncSitePlan="Yes",2500+150*NTotal+IF(NDcfc&gt;0,1000,0),0)</f>
@@ -7211,7 +7314,7 @@
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>173</v>
+        <v>180</v>
       </c>
       <c r="B35" s="9">
         <f>IF(IncSLD="Yes",IF(NDcfc&gt;0,6000+900*NDcfc+150*NumL2,2500+150*NumL2),0)</f>
@@ -7219,7 +7322,7 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>174</v>
+        <v>181</v>
       </c>
       <c r="B36" s="9">
         <f>C36*PmRate</f>
@@ -7230,7 +7333,7 @@
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
       <c r="B37" s="9">
         <f>IF(IncPermits="Yes",IF(NDcfc&gt;0,500+0.02*Valuation,300),0)</f>
@@ -7238,7 +7341,7 @@
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
-        <v>176</v>
+        <v>183</v>
       </c>
       <c r="B38" s="9">
         <f>SUM(B34:B37)</f>
@@ -7246,7 +7349,7 @@
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="13" t="s">
-        <v>177</v>
+        <v>184</v>
       </c>
       <c r="B40" s="14">
         <f>ConstructionTotal+LaborCost+B23+B27+B28+B29+B30+B31+B38</f>
@@ -7254,7 +7357,7 @@
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>178</v>
+        <v>185</v>
       </c>
       <c r="B41" s="9">
         <f>-RebateAmt</f>
@@ -7262,7 +7365,7 @@
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" s="16" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="B42" s="32">
         <f>TotalCost-RebateAmt</f>
@@ -7297,27 +7400,27 @@
   <sheetData>
     <row r="2" ht="15.75" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B2" s="33" t="s">
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="C2" s="34" t="s">
-        <v>180</v>
+        <v>187</v>
       </c>
       <c r="D2" s="35" t="s">
-        <v>181</v>
+        <v>188</v>
       </c>
       <c r="E2" s="36" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="F2" s="35" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="G2" s="37" t="s">
-        <v>183</v>
+        <v>190</v>
       </c>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="38" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="C3" s="39">
         <v>1</v>
@@ -7335,13 +7438,13 @@
         <f>F3*C3</f>
       </c>
       <c r="J3" s="43" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="K3" s="44"/>
     </row>
     <row r="4" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B4" s="38" t="s">
-        <v>186</v>
+        <v>193</v>
       </c>
       <c r="C4" s="39">
         <v>1</v>
@@ -7359,15 +7462,15 @@
         <f>F4*C4</f>
       </c>
       <c r="J4" s="45" t="s">
-        <v>187</v>
+        <v>194</v>
       </c>
       <c r="K4" s="46">
-        <f>LaborDayRate</f>
+        <f>IF(LaborDays&gt;0,LaborBase/LaborDays,0)</f>
       </c>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B5" s="38" t="s">
-        <v>188</v>
+        <v>195</v>
       </c>
       <c r="C5" s="39">
         <v>1</v>
@@ -7385,7 +7488,7 @@
         <f>F5*C5</f>
       </c>
       <c r="J5" s="45" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="K5" s="47">
         <f>LaborDays</f>
@@ -7393,7 +7496,7 @@
     </row>
     <row r="6" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B6" s="38" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="C6" s="39">
         <v>1</v>
@@ -7411,7 +7514,7 @@
         <f>F6*C6</f>
       </c>
       <c r="J6" s="45" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="K6" s="47">
         <f>K5/30</f>
@@ -7419,7 +7522,7 @@
     </row>
     <row r="7" ht="15.75" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B7" s="38" t="s">
-        <v>192</v>
+        <v>199</v>
       </c>
       <c r="C7" s="39">
         <v>1</v>
@@ -7437,7 +7540,7 @@
         <f>F7*C7</f>
       </c>
       <c r="J7" s="48" t="s">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="K7" s="49">
         <f>K5*K4</f>
@@ -7445,7 +7548,7 @@
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B8" s="38" t="s">
-        <v>194</v>
+        <v>201</v>
       </c>
       <c r="C8" s="39">
         <v>1</v>
@@ -7465,7 +7568,7 @@
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B9" s="38" t="s">
-        <v>195</v>
+        <v>202</v>
       </c>
       <c r="C9" s="39">
         <v>1</v>
@@ -7485,7 +7588,7 @@
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B10" s="38" t="s">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="C10" s="39">
         <v>1</v>
@@ -7505,7 +7608,7 @@
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B11" s="38" t="s">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="C11" s="39">
         <v>1</v>
@@ -7545,7 +7648,7 @@
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B13" s="38" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="C13" s="39">
         <v>1</v>
@@ -7565,7 +7668,7 @@
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B14" s="38" t="s">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="C14" s="39">
         <v>1</v>
@@ -7596,7 +7699,7 @@
     <row r="16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" ht="15.75" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B17" s="55" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="C17" s="55"/>
       <c r="D17" s="55"/>
@@ -7606,7 +7709,7 @@
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B18" s="38" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="C18" s="39">
         <f>K5</f>
@@ -7637,7 +7740,7 @@
     <row r="20" ht="15.75" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B20" s="48"/>
       <c r="C20" s="56" t="s">
-        <v>183</v>
+        <v>190</v>
       </c>
       <c r="D20" s="56"/>
       <c r="E20" s="56"/>
@@ -7668,12 +7771,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="15" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="B3">
         <f>NTotal</f>
@@ -7681,7 +7784,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>203</v>
+        <v>210</v>
       </c>
       <c r="B4">
         <f>IF(NTotal&lt;=0,0,IF(NTotal&lt;=100,1,1+ROUNDUP((NTotal-100)/300,0)))</f>
@@ -7689,7 +7792,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>204</v>
+        <v>211</v>
       </c>
       <c r="B5">
         <f>IF(NTotal&lt;=4,0,IF(NTotal&lt;=50,1,IF(NTotal&lt;=75,2,IF(NTotal&lt;=100,3,3+ROUNDUP((NTotal-100)/60,0)))))</f>
@@ -7697,7 +7800,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>205</v>
+        <v>212</v>
       </c>
       <c r="B6">
         <f>IF(NTotal&lt;=25,0,IF(NTotal&lt;=50,1,IF(NTotal&lt;=75,2,IF(NTotal&lt;=100,3,3+ROUNDUP((NTotal-100)/50,0)))))</f>
@@ -7705,7 +7808,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>206</v>
+        <v>213</v>
       </c>
       <c r="B7">
         <f>AdaVan+AdaStd+AdaAmb</f>
@@ -7713,7 +7816,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>207</v>
+        <v>214</v>
       </c>
       <c r="B9">
         <f>VLOOKUP(Terrain,TerrainTable,4,FALSE)</f>
@@ -7721,7 +7824,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>208</v>
+        <v>215</v>
       </c>
       <c r="B10" s="9">
         <f>(AdaVan*AdaVanCost+AdaStd*AdaStdCost+AdaAmb*AdaAmbCost)*VLOOKUP(Terrain,TerrainTable,4,FALSE)+IF(NTotal&gt;0,AdaRampCost,0)</f>
@@ -7729,130 +7832,130 @@
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>209</v>
+        <v>216</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="58" t="s">
-        <v>210</v>
+        <v>217</v>
       </c>
       <c r="B14" s="58" t="s">
-        <v>211</v>
+        <v>218</v>
       </c>
       <c r="C14" s="58" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="D14" s="58" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="59" t="s">
-        <v>214</v>
+        <v>221</v>
       </c>
       <c r="B15" s="59" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="C15" s="59" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
       <c r="D15" s="59" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="59" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="B16" s="59" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="C16" s="59" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="D16" s="59" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="59" t="s">
-        <v>218</v>
+        <v>225</v>
       </c>
       <c r="B17" s="59" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="C17" s="59" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="D17" s="59" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="59" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
       <c r="B18" s="59" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="C18" s="59" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="D18" s="59" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="59" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="B19" s="59" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="C19" s="59" t="s">
-        <v>222</v>
+        <v>229</v>
       </c>
       <c r="D19" s="59" t="s">
-        <v>222</v>
+        <v>229</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="59" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
       <c r="B20" s="59" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
       <c r="C20" s="59" t="s">
-        <v>225</v>
+        <v>232</v>
       </c>
       <c r="D20" s="59" t="s">
-        <v>226</v>
+        <v>233</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" s="60" t="s">
-        <v>227</v>
+        <v>234</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" s="60" t="s">
-        <v>228</v>
+        <v>235</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="60" t="s">
-        <v>229</v>
+        <v>236</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" s="60" t="s">
-        <v>230</v>
+        <v>237</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" s="60" t="s">
-        <v>231</v>
+        <v>238</v>
       </c>
     </row>
   </sheetData>
@@ -7873,26 +7976,26 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="15" t="s">
-        <v>232</v>
+        <v>239</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>233</v>
+        <v>240</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>234</v>
+        <v>241</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>237</v>
+        <v>244</v>
       </c>
       <c r="B4">
         <f>2</f>
@@ -7901,12 +8004,12 @@
         <f>4</f>
       </c>
       <c r="D4" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="B5">
         <f>IF(IncSitePlan="Yes",5+ROUNDUP(NTotal/4,0),0)</f>
@@ -7915,12 +8018,12 @@
         <f>IF(IncSitePlan="Yes",10+ROUNDUP(NTotal/4,0),0)</f>
       </c>
       <c r="D5" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="B6">
         <f>IF(IncSLD="Yes",IF(NDcfc&gt;0,10+ROUNDUP(NDcfc/2,0),7),0)</f>
@@ -7929,12 +8032,12 @@
         <f>IF(IncSLD="Yes",IF(NDcfc&gt;0,17+ROUNDUP(NDcfc/2,0),14),0)</f>
       </c>
       <c r="D6" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>240</v>
+        <v>247</v>
       </c>
       <c r="B7">
         <f>IF(IncPermits="Yes",IF(NDcfc&gt;0,20,5),0)</f>
@@ -7943,12 +8046,12 @@
         <f>IF(IncPermits="Yes",IF(NDcfc&gt;0,60,15),0)</f>
       </c>
       <c r="D7" t="s">
-        <v>241</v>
+        <v>248</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>242</v>
+        <v>249</v>
       </c>
       <c r="B8">
         <f>IF(NDcfc&gt;0,85,20)</f>
@@ -7957,12 +8060,12 @@
         <f>IF(NDcfc&gt;0,250,60)</f>
       </c>
       <c r="D8" t="s">
-        <v>243</v>
+        <v>250</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>244</v>
+        <v>251</v>
       </c>
       <c r="B9">
         <f>LaborDays</f>
@@ -7971,12 +8074,12 @@
         <f>LaborDays+7</f>
       </c>
       <c r="D9" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>245</v>
+        <v>252</v>
       </c>
       <c r="B10">
         <f>5</f>
@@ -7985,12 +8088,12 @@
         <f>10</f>
       </c>
       <c r="D10" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="B12">
         <f>MAX(B4+B5+B6+B7+B9+B10,B8)</f>
@@ -8001,7 +8104,7 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="B13">
         <f>ROUND(B12/21,1)</f>
@@ -8039,7 +8142,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="15" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.25">
@@ -8050,40 +8153,40 @@
         <v>20</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>249</v>
+        <v>256</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>21</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>250</v>
+        <v>257</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
       <c r="I3" s="7" t="s">
-        <v>252</v>
+        <v>259</v>
       </c>
       <c r="J3" s="7" t="s">
-        <v>253</v>
+        <v>260</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>254</v>
+        <v>261</v>
       </c>
       <c r="L3" s="7" t="s">
-        <v>255</v>
+        <v>262</v>
       </c>
       <c r="M3" s="7" t="s">
         <v>44</v>
       </c>
       <c r="N3" s="7" t="s">
-        <v>256</v>
+        <v>263</v>
       </c>
       <c r="O3" s="7" t="s">
         <v>42</v>
@@ -8092,21 +8195,21 @@
         <v>35</v>
       </c>
       <c r="R3" s="7" t="s">
-        <v>257</v>
+        <v>264</v>
       </c>
       <c r="S3" s="7" t="s">
-        <v>258</v>
+        <v>265</v>
       </c>
       <c r="T3" s="7" t="s">
-        <v>259</v>
+        <v>266</v>
       </c>
       <c r="U3" s="7" t="s">
-        <v>260</v>
+        <v>267</v>
       </c>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>261</v>
+        <v>268</v>
       </c>
       <c r="B4" s="61">
         <v>3000</v>
@@ -8115,7 +8218,7 @@
         <v>538</v>
       </c>
       <c r="D4" t="s">
-        <v>262</v>
+        <v>269</v>
       </c>
       <c r="E4">
         <v>208</v>
@@ -8145,10 +8248,10 @@
         <v>2</v>
       </c>
       <c r="N4" t="s">
-        <v>263</v>
+        <v>270</v>
       </c>
       <c r="O4" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="Q4" t="s">
         <v>36</v>
@@ -8168,7 +8271,7 @@
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
       <c r="B5" s="61">
         <v>3500</v>
@@ -8177,7 +8280,7 @@
         <v>532</v>
       </c>
       <c r="D5" t="s">
-        <v>262</v>
+        <v>269</v>
       </c>
       <c r="E5">
         <v>208</v>
@@ -8207,13 +8310,13 @@
         <v>2</v>
       </c>
       <c r="N5" t="s">
-        <v>263</v>
+        <v>270</v>
       </c>
       <c r="O5" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="Q5" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="R5" s="8">
         <v>1.2</v>
@@ -8239,7 +8342,7 @@
         <v>542</v>
       </c>
       <c r="D6" t="s">
-        <v>262</v>
+        <v>269</v>
       </c>
       <c r="E6">
         <v>208</v>
@@ -8269,13 +8372,13 @@
         <v>2</v>
       </c>
       <c r="N6" t="s">
-        <v>263</v>
+        <v>270</v>
       </c>
       <c r="O6" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="Q6" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="R6" s="8">
         <v>1.5</v>
@@ -8292,7 +8395,7 @@
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="B7" s="61">
         <v>5000</v>
@@ -8301,7 +8404,7 @@
         <v>611</v>
       </c>
       <c r="D7" t="s">
-        <v>262</v>
+        <v>269</v>
       </c>
       <c r="E7">
         <v>208</v>
@@ -8331,13 +8434,13 @@
         <v>2</v>
       </c>
       <c r="N7" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="O7" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="Q7" t="s">
-        <v>270</v>
+        <v>277</v>
       </c>
       <c r="R7" s="8">
         <v>2.5</v>
@@ -8354,7 +8457,7 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>271</v>
+        <v>278</v>
       </c>
       <c r="B8" s="61">
         <v>7500</v>
@@ -8363,7 +8466,7 @@
         <v>943</v>
       </c>
       <c r="D8" t="s">
-        <v>262</v>
+        <v>269</v>
       </c>
       <c r="E8">
         <v>208</v>
@@ -8393,15 +8496,15 @@
         <v>2</v>
       </c>
       <c r="N8" t="s">
-        <v>272</v>
+        <v>279</v>
       </c>
       <c r="O8" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B9" s="61">
         <v>5500</v>
@@ -8410,7 +8513,7 @@
         <v>693</v>
       </c>
       <c r="D9" t="s">
-        <v>262</v>
+        <v>269</v>
       </c>
       <c r="E9">
         <v>208</v>
@@ -8440,15 +8543,15 @@
         <v>2</v>
       </c>
       <c r="N9" t="s">
-        <v>263</v>
+        <v>270</v>
       </c>
       <c r="O9" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>274</v>
+        <v>281</v>
       </c>
       <c r="B10" s="61">
         <v>6500</v>
@@ -8457,7 +8560,7 @@
         <v>710</v>
       </c>
       <c r="D10" t="s">
-        <v>262</v>
+        <v>269</v>
       </c>
       <c r="E10">
         <v>208</v>
@@ -8487,13 +8590,13 @@
         <v>2</v>
       </c>
       <c r="N10" t="s">
-        <v>263</v>
+        <v>270</v>
       </c>
       <c r="O10" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="Q10" t="s">
-        <v>275</v>
+        <v>282</v>
       </c>
       <c r="R10" s="61">
         <v>40.81</v>
@@ -8501,7 +8604,7 @@
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>276</v>
+        <v>283</v>
       </c>
       <c r="B11" s="61">
         <v>8500</v>
@@ -8510,7 +8613,7 @@
         <v>862</v>
       </c>
       <c r="D11" t="s">
-        <v>262</v>
+        <v>269</v>
       </c>
       <c r="E11">
         <v>208</v>
@@ -8540,13 +8643,13 @@
         <v>2</v>
       </c>
       <c r="N11" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="O11" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="Q11" t="s">
-        <v>277</v>
+        <v>284</v>
       </c>
       <c r="R11" s="62">
         <v>0.1</v>
@@ -8554,7 +8657,7 @@
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>278</v>
+        <v>285</v>
       </c>
       <c r="B12" s="61">
         <v>32000</v>
@@ -8563,7 +8666,7 @@
         <v>654</v>
       </c>
       <c r="D12" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="E12">
         <v>480</v>
@@ -8593,13 +8696,13 @@
         <v>3</v>
       </c>
       <c r="N12" t="s">
-        <v>280</v>
+        <v>287</v>
       </c>
       <c r="O12" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="Q12" t="s">
-        <v>281</v>
+        <v>288</v>
       </c>
       <c r="R12" s="62">
         <v>0.0725</v>
@@ -8607,7 +8710,7 @@
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>282</v>
+        <v>289</v>
       </c>
       <c r="B13" s="61">
         <v>35000</v>
@@ -8616,7 +8719,7 @@
         <v>654</v>
       </c>
       <c r="D13" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="E13">
         <v>480</v>
@@ -8646,13 +8749,13 @@
         <v>3</v>
       </c>
       <c r="N13" t="s">
-        <v>280</v>
+        <v>287</v>
       </c>
       <c r="O13" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="Q13" t="s">
-        <v>283</v>
+        <v>290</v>
       </c>
       <c r="R13" s="61">
         <v>2250</v>
@@ -8660,7 +8763,7 @@
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>284</v>
+        <v>291</v>
       </c>
       <c r="B14" s="61">
         <v>38000</v>
@@ -8669,7 +8772,7 @@
         <v>657</v>
       </c>
       <c r="D14" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="E14">
         <v>480</v>
@@ -8699,13 +8802,13 @@
         <v>3</v>
       </c>
       <c r="N14" t="s">
-        <v>280</v>
+        <v>287</v>
       </c>
       <c r="O14" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="Q14" t="s">
-        <v>285</v>
+        <v>292</v>
       </c>
       <c r="R14" s="61">
         <v>358</v>
@@ -8713,7 +8816,7 @@
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>286</v>
+        <v>293</v>
       </c>
       <c r="B15" s="61">
         <v>42000</v>
@@ -8722,7 +8825,7 @@
         <v>657</v>
       </c>
       <c r="D15" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="E15">
         <v>480</v>
@@ -8752,13 +8855,13 @@
         <v>3</v>
       </c>
       <c r="N15" t="s">
-        <v>280</v>
+        <v>287</v>
       </c>
       <c r="O15" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="Q15" t="s">
-        <v>287</v>
+        <v>294</v>
       </c>
       <c r="R15" s="62">
         <v>0.05</v>
@@ -8766,7 +8869,7 @@
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>288</v>
+        <v>295</v>
       </c>
       <c r="B16" s="61">
         <v>52000</v>
@@ -8775,7 +8878,7 @@
         <v>768</v>
       </c>
       <c r="D16" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="E16">
         <v>480</v>
@@ -8805,13 +8908,13 @@
         <v>3</v>
       </c>
       <c r="N16" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="O16" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="Q16" t="s">
-        <v>290</v>
+        <v>297</v>
       </c>
       <c r="R16" s="61">
         <v>1500</v>
@@ -8819,7 +8922,7 @@
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B17" s="61">
         <v>57000</v>
@@ -8828,7 +8931,7 @@
         <v>768</v>
       </c>
       <c r="D17" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="E17">
         <v>480</v>
@@ -8858,13 +8961,13 @@
         <v>3</v>
       </c>
       <c r="N17" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="O17" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="Q17" t="s">
-        <v>292</v>
+        <v>299</v>
       </c>
       <c r="R17" s="8">
         <v>2000</v>
@@ -8872,7 +8975,7 @@
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>293</v>
+        <v>300</v>
       </c>
       <c r="B18" s="61">
         <v>60000</v>
@@ -8881,7 +8984,7 @@
         <v>808</v>
       </c>
       <c r="D18" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="E18">
         <v>480</v>
@@ -8911,13 +9014,13 @@
         <v>3</v>
       </c>
       <c r="N18" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="O18" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="Q18" t="s">
-        <v>294</v>
+        <v>301</v>
       </c>
       <c r="R18" s="61">
         <v>6500</v>
@@ -8925,7 +9028,7 @@
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>295</v>
+        <v>302</v>
       </c>
       <c r="B19" s="61">
         <v>66000</v>
@@ -8934,7 +9037,7 @@
         <v>808</v>
       </c>
       <c r="D19" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="E19">
         <v>480</v>
@@ -8964,13 +9067,13 @@
         <v>3</v>
       </c>
       <c r="N19" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="O19" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="Q19" t="s">
-        <v>296</v>
+        <v>303</v>
       </c>
       <c r="R19" s="61">
         <v>4900</v>
@@ -8978,7 +9081,7 @@
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>297</v>
+        <v>304</v>
       </c>
       <c r="B20" s="61">
         <v>72000</v>
@@ -8987,7 +9090,7 @@
         <v>1003</v>
       </c>
       <c r="D20" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="E20">
         <v>480</v>
@@ -9017,13 +9120,13 @@
         <v>3</v>
       </c>
       <c r="N20" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
       <c r="O20" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="Q20" t="s">
-        <v>299</v>
+        <v>306</v>
       </c>
       <c r="R20" s="61">
         <v>3500</v>
@@ -9031,7 +9134,7 @@
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>300</v>
+        <v>307</v>
       </c>
       <c r="B21" s="61">
         <v>79000</v>
@@ -9040,7 +9143,7 @@
         <v>1003</v>
       </c>
       <c r="D21" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="E21">
         <v>480</v>
@@ -9070,13 +9173,13 @@
         <v>3</v>
       </c>
       <c r="N21" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
       <c r="O21" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="Q21" t="s">
-        <v>301</v>
+        <v>308</v>
       </c>
       <c r="R21" s="61">
         <v>5200</v>
@@ -9084,7 +9187,7 @@
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>302</v>
+        <v>309</v>
       </c>
       <c r="B22" s="61">
         <v>80000</v>
@@ -9093,7 +9196,7 @@
         <v>1086</v>
       </c>
       <c r="D22" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="E22">
         <v>480</v>
@@ -9123,13 +9226,13 @@
         <v>3</v>
       </c>
       <c r="N22" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
       <c r="O22" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="Q22" t="s">
-        <v>303</v>
+        <v>310</v>
       </c>
       <c r="R22" s="61">
         <v>2903</v>
@@ -9137,7 +9240,7 @@
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>304</v>
+        <v>311</v>
       </c>
       <c r="B23" s="61">
         <v>88000</v>
@@ -9146,7 +9249,7 @@
         <v>1086</v>
       </c>
       <c r="D23" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="E23">
         <v>480</v>
@@ -9176,13 +9279,13 @@
         <v>3</v>
       </c>
       <c r="N23" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
       <c r="O23" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="Q23" t="s">
-        <v>305</v>
+        <v>312</v>
       </c>
       <c r="R23" s="61">
         <v>758</v>
@@ -9199,7 +9302,7 @@
         <v>1182</v>
       </c>
       <c r="D24" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="E24">
         <v>480</v>
@@ -9229,13 +9332,13 @@
         <v>3</v>
       </c>
       <c r="N24" t="s">
-        <v>306</v>
+        <v>313</v>
       </c>
       <c r="O24" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="Q24" t="s">
-        <v>307</v>
+        <v>314</v>
       </c>
       <c r="R24" s="61">
         <v>302</v>
@@ -9243,7 +9346,7 @@
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>308</v>
+        <v>315</v>
       </c>
       <c r="B25" s="61">
         <v>100000</v>
@@ -9252,7 +9355,7 @@
         <v>1182</v>
       </c>
       <c r="D25" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="E25">
         <v>480</v>
@@ -9282,13 +9385,13 @@
         <v>3</v>
       </c>
       <c r="N25" t="s">
-        <v>306</v>
+        <v>313</v>
       </c>
       <c r="O25" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="Q25" t="s">
-        <v>309</v>
+        <v>316</v>
       </c>
       <c r="R25" s="61">
         <v>658</v>
@@ -9296,7 +9399,7 @@
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="B26" s="61">
         <v>105000</v>
@@ -9305,7 +9408,7 @@
         <v>1518</v>
       </c>
       <c r="D26" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="E26">
         <v>480</v>
@@ -9335,13 +9438,13 @@
         <v>3</v>
       </c>
       <c r="N26" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="O26" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="Q26" t="s">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="R26" s="61">
         <v>396</v>
@@ -9349,7 +9452,7 @@
     </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>312</v>
+        <v>319</v>
       </c>
       <c r="B27" s="61">
         <v>115000</v>
@@ -9358,7 +9461,7 @@
         <v>1518</v>
       </c>
       <c r="D27" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="E27">
         <v>480</v>
@@ -9388,13 +9491,13 @@
         <v>3</v>
       </c>
       <c r="N27" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="O27" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="Q27" t="s">
-        <v>313</v>
+        <v>320</v>
       </c>
       <c r="R27" s="61">
         <v>5000</v>
@@ -9402,7 +9505,7 @@
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>314</v>
+        <v>321</v>
       </c>
       <c r="B28" s="61">
         <v>120000</v>
@@ -9411,7 +9514,7 @@
         <v>1816</v>
       </c>
       <c r="D28" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="E28">
         <v>480</v>
@@ -9441,13 +9544,13 @@
         <v>3</v>
       </c>
       <c r="N28" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="O28" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="Q28" t="s">
-        <v>316</v>
+        <v>323</v>
       </c>
       <c r="R28" s="61">
         <v>1500</v>
@@ -9455,7 +9558,7 @@
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>317</v>
+        <v>324</v>
       </c>
       <c r="B29" s="61">
         <v>130000</v>
@@ -9464,7 +9567,7 @@
         <v>1816</v>
       </c>
       <c r="D29" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="E29">
         <v>480</v>
@@ -9494,13 +9597,13 @@
         <v>3</v>
       </c>
       <c r="N29" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="O29" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="Q29" t="s">
-        <v>318</v>
+        <v>325</v>
       </c>
       <c r="R29" s="61">
         <v>250</v>
@@ -9508,7 +9611,7 @@
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>319</v>
+        <v>326</v>
       </c>
       <c r="B30" s="61">
         <v>135000</v>
@@ -9517,7 +9620,7 @@
         <v>1816</v>
       </c>
       <c r="D30" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="E30">
         <v>480</v>
@@ -9547,13 +9650,13 @@
         <v>3</v>
       </c>
       <c r="N30" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="O30" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="Q30" t="s">
-        <v>320</v>
+        <v>327</v>
       </c>
       <c r="R30" s="61">
         <v>3519</v>
@@ -9561,7 +9664,7 @@
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>321</v>
+        <v>328</v>
       </c>
       <c r="B31" s="61">
         <v>147000</v>
@@ -9570,7 +9673,7 @@
         <v>1816</v>
       </c>
       <c r="D31" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="E31">
         <v>480</v>
@@ -9600,13 +9703,13 @@
         <v>3</v>
       </c>
       <c r="N31" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="O31" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="Q31" t="s">
-        <v>322</v>
+        <v>329</v>
       </c>
       <c r="R31" s="61">
         <v>261</v>
@@ -9614,7 +9717,7 @@
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>323</v>
+        <v>330</v>
       </c>
       <c r="B32" s="61">
         <v>155000</v>
@@ -9623,7 +9726,7 @@
         <v>2007</v>
       </c>
       <c r="D32" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="E32">
         <v>480</v>
@@ -9656,12 +9759,12 @@
         <v>54</v>
       </c>
       <c r="O32" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>324</v>
+        <v>331</v>
       </c>
       <c r="B33" s="61">
         <v>168000</v>
@@ -9670,7 +9773,7 @@
         <v>2007</v>
       </c>
       <c r="D33" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="E33">
         <v>480</v>
@@ -9703,25 +9806,25 @@
         <v>54</v>
       </c>
       <c r="O33" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>325</v>
+        <v>332</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="7" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>328</v>
+        <v>335</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
@@ -9806,15 +9909,15 @@
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" s="7" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
       <c r="B50" s="7" t="s">
-        <v>328</v>
+        <v>335</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
@@ -9867,15 +9970,15 @@
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
-        <v>330</v>
+        <v>337</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" s="7" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
       <c r="B59" s="7" t="s">
-        <v>328</v>
+        <v>335</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.25">
@@ -9936,15 +10039,15 @@
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" s="3" t="s">
-        <v>331</v>
+        <v>338</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
       <c r="B69" s="7" t="s">
-        <v>328</v>
+        <v>335</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.25">
@@ -10045,15 +10148,15 @@
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A83" s="3" t="s">
-        <v>332</v>
+        <v>339</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84" s="7" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
       <c r="B84" s="7" t="s">
-        <v>328</v>
+        <v>335</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.25">
@@ -10082,7 +10185,7 @@
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A89" s="3" t="s">
-        <v>333</v>
+        <v>340</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.25">
@@ -10267,29 +10370,29 @@
     </row>
     <row r="127" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A127" s="3" t="s">
-        <v>334</v>
+        <v>341</v>
       </c>
     </row>
     <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128" s="7" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
       <c r="B128" s="7" t="s">
-        <v>335</v>
+        <v>342</v>
       </c>
       <c r="C128" s="7" t="s">
-        <v>336</v>
+        <v>343</v>
       </c>
       <c r="D128" s="7" t="s">
-        <v>337</v>
+        <v>344</v>
       </c>
       <c r="E128" s="7" t="s">
-        <v>338</v>
+        <v>345</v>
       </c>
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>339</v>
+        <v>346</v>
       </c>
       <c r="B129" s="61">
         <v>0</v>
@@ -10306,7 +10409,7 @@
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>340</v>
+        <v>347</v>
       </c>
       <c r="B130" s="61">
         <v>0</v>
@@ -10323,7 +10426,7 @@
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>341</v>
+        <v>348</v>
       </c>
       <c r="B131" s="61">
         <v>0.30329</v>
@@ -10340,7 +10443,7 @@
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>342</v>
+        <v>349</v>
       </c>
       <c r="B132" s="61">
         <v>0.56613</v>
@@ -10357,7 +10460,7 @@
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>263</v>
+        <v>270</v>
       </c>
       <c r="B133" s="61">
         <v>0.87104</v>
@@ -10374,7 +10477,7 @@
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="B134" s="61">
         <v>1.33293</v>
@@ -10391,7 +10494,7 @@
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="B135" s="61">
         <v>1.68126</v>
@@ -10408,7 +10511,7 @@
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>344</v>
+        <v>351</v>
       </c>
       <c r="B136" s="61">
         <v>2.1044</v>
@@ -10425,7 +10528,7 @@
     </row>
     <row r="137" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>272</v>
+        <v>279</v>
       </c>
       <c r="B137" s="61">
         <v>2.39833</v>
@@ -10442,7 +10545,7 @@
     </row>
     <row r="138" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>280</v>
+        <v>287</v>
       </c>
       <c r="B138" s="61">
         <v>2.95304</v>
@@ -10459,7 +10562,7 @@
     </row>
     <row r="139" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>345</v>
+        <v>352</v>
       </c>
       <c r="B139" s="61">
         <v>3.63758</v>
@@ -10476,7 +10579,7 @@
     </row>
     <row r="140" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="B140" s="61">
         <v>4.5658</v>
@@ -10510,7 +10613,7 @@
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="B142" s="61">
         <v>6.64016</v>
@@ -10527,7 +10630,7 @@
     </row>
     <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
       <c r="B143" s="61">
         <v>7.9632</v>
@@ -10561,7 +10664,7 @@
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>306</v>
+        <v>313</v>
       </c>
       <c r="B145" s="61">
         <v>10.60671</v>
@@ -10578,7 +10681,7 @@
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B146" s="61">
         <v>11.334</v>
@@ -10595,7 +10698,7 @@
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>347</v>
+        <v>354</v>
       </c>
       <c r="B147" s="61">
         <v>13.30059</v>
@@ -10629,7 +10732,7 @@
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>348</v>
+        <v>355</v>
       </c>
       <c r="B149" s="61">
         <v>0</v>
@@ -10646,7 +10749,7 @@
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>349</v>
+        <v>356</v>
       </c>
       <c r="B150" s="61">
         <v>25.921</v>
@@ -10663,7 +10766,7 @@
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>350</v>
+        <v>357</v>
       </c>
       <c r="B151" s="61">
         <v>0</v>
@@ -10680,7 +10783,7 @@
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>351</v>
+        <v>358</v>
       </c>
       <c r="B152" s="61">
         <v>0</v>
@@ -10697,7 +10800,7 @@
     </row>
     <row r="153" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>352</v>
+        <v>359</v>
       </c>
       <c r="B153" s="61">
         <v>34.398</v>
@@ -10714,7 +10817,7 @@
     </row>
     <row r="154" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A154" s="2" t="s">
-        <v>353</v>
+        <v>360</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Template: tie Costs Internal rows to the app (GPR bucket, data box)
Filling the same intake in the app and the template gave different
Costs Internal rows. Two causes, both template-side:

- GPR scan was mapped into the Utility row; the app books it as a
  peripherals custom item, i.e. the Wires/Conduits/Peripherals row.
  Utility was overstated by the scan cost ($1,500 at defaults).
- The site's single data box ($1,500) was smeared into the per-charger
  install allowance during calibration ($1,500/6 per unit), so an
  11-charger site carried $2,750 of data box. Now excluded from the
  allowance and priced once per site (DataBoxCost scalar, Estimate B7).

verify-template.py now asserts every Costs Internal row against the
app engine's golden values (exact for formula rows, ±2% for the two
calibrated allowance rows). Template mirror delta: 0.2% -> 0.0%.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/RFC-Template.xlsx
+++ b/templates/RFC-Template.xlsx
@@ -41,39 +41,40 @@
     <definedName name="CpmPct">RateCard!$R$15</definedName>
     <definedName name="GprDayRate">RateCard!$R$16</definedName>
     <definedName name="GprFtPerDay">RateCard!$R$17</definedName>
-    <definedName name="AdaVanCost">RateCard!$R$18</definedName>
-    <definedName name="AdaStdCost">RateCard!$R$19</definedName>
-    <definedName name="AdaAmbCost">RateCard!$R$20</definedName>
-    <definedName name="AdaRampCost">RateCard!$R$21</definedName>
-    <definedName name="ConcreteRate">RateCard!$R$22</definedName>
-    <definedName name="ShortLoadFee">RateCard!$R$23</definedName>
-    <definedName name="AsphaltRate">RateCard!$R$24</definedName>
-    <definedName name="StallSqFt">RateCard!$R$25</definedName>
-    <definedName name="BollardCost">RateCard!$R$26</definedName>
-    <definedName name="BollardPerChg">RateCard!$R$27</definedName>
-    <definedName name="BollardAtGear">RateCard!$R$28</definedName>
-    <definedName name="BollardAtStepdown">RateCard!$R$29</definedName>
-    <definedName name="ConsumDcfc">RateCard!$R$30</definedName>
-    <definedName name="ConsumL2">RateCard!$R$31</definedName>
-    <definedName name="PadYdDcfc">RateCard!$R$32</definedName>
-    <definedName name="PadYdL2">RateCard!$R$33</definedName>
-    <definedName name="PadYdGear">RateCard!$R$34</definedName>
-    <definedName name="PadYdXfmr">RateCard!$R$35</definedName>
-    <definedName name="PadYdBollard">RateCard!$R$36</definedName>
-    <definedName name="TransformerPad">RateCard!$R$37</definedName>
-    <definedName name="CommDcfc">RateCard!$R$38</definedName>
-    <definedName name="CommL2">RateCard!$R$39</definedName>
-    <definedName name="EquipBase">RateCard!$R$40</definedName>
-    <definedName name="EquipPerDay">RateCard!$R$41</definedName>
-    <definedName name="EquipBaseEmt">RateCard!$R$42</definedName>
-    <definedName name="EquipPerDayEmt">RateCard!$R$43</definedName>
-    <definedName name="EmtRackCost">RateCard!$R$44</definedName>
-    <definedName name="EmtStrapCost">RateCard!$R$45</definedName>
-    <definedName name="EmtFtPerDay">RateCard!$R$46</definedName>
-    <definedName name="PermitBase">RateCard!$R$47</definedName>
-    <definedName name="PermitPerChg">RateCard!$R$48</definedName>
-    <definedName name="UtilAppDcfc">RateCard!$R$49</definedName>
-    <definedName name="UtilAppL2">RateCard!$R$50</definedName>
+    <definedName name="DataBoxCost">RateCard!$R$18</definedName>
+    <definedName name="AdaVanCost">RateCard!$R$19</definedName>
+    <definedName name="AdaStdCost">RateCard!$R$20</definedName>
+    <definedName name="AdaAmbCost">RateCard!$R$21</definedName>
+    <definedName name="AdaRampCost">RateCard!$R$22</definedName>
+    <definedName name="ConcreteRate">RateCard!$R$23</definedName>
+    <definedName name="ShortLoadFee">RateCard!$R$24</definedName>
+    <definedName name="AsphaltRate">RateCard!$R$25</definedName>
+    <definedName name="StallSqFt">RateCard!$R$26</definedName>
+    <definedName name="BollardCost">RateCard!$R$27</definedName>
+    <definedName name="BollardPerChg">RateCard!$R$28</definedName>
+    <definedName name="BollardAtGear">RateCard!$R$29</definedName>
+    <definedName name="BollardAtStepdown">RateCard!$R$30</definedName>
+    <definedName name="ConsumDcfc">RateCard!$R$31</definedName>
+    <definedName name="ConsumL2">RateCard!$R$32</definedName>
+    <definedName name="PadYdDcfc">RateCard!$R$33</definedName>
+    <definedName name="PadYdL2">RateCard!$R$34</definedName>
+    <definedName name="PadYdGear">RateCard!$R$35</definedName>
+    <definedName name="PadYdXfmr">RateCard!$R$36</definedName>
+    <definedName name="PadYdBollard">RateCard!$R$37</definedName>
+    <definedName name="TransformerPad">RateCard!$R$38</definedName>
+    <definedName name="CommDcfc">RateCard!$R$39</definedName>
+    <definedName name="CommL2">RateCard!$R$40</definedName>
+    <definedName name="EquipBase">RateCard!$R$41</definedName>
+    <definedName name="EquipPerDay">RateCard!$R$42</definedName>
+    <definedName name="EquipBaseEmt">RateCard!$R$43</definedName>
+    <definedName name="EquipPerDayEmt">RateCard!$R$44</definedName>
+    <definedName name="EmtRackCost">RateCard!$R$45</definedName>
+    <definedName name="EmtStrapCost">RateCard!$R$46</definedName>
+    <definedName name="EmtFtPerDay">RateCard!$R$47</definedName>
+    <definedName name="PermitBase">RateCard!$R$48</definedName>
+    <definedName name="PermitPerChg">RateCard!$R$49</definedName>
+    <definedName name="UtilAppDcfc">RateCard!$R$50</definedName>
+    <definedName name="UtilAppL2">RateCard!$R$51</definedName>
     <definedName name="NTotal">Intake!$B$36</definedName>
     <definedName name="NDcfc">Intake!$B$37</definedName>
     <definedName name="NumL2">Intake!$B$38</definedName>
@@ -122,7 +123,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="788" uniqueCount="471">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="789" uniqueCount="472">
   <si>
     <t>RFC INTAKE — EV Charging Project</t>
   </si>
@@ -637,7 +638,7 @@
     <t>Electrical supply &amp; construction</t>
   </si>
   <si>
-    <t>Wire runs (Takeoff + feeders) + conduit &amp; install allowance</t>
+    <t>Wire runs (Takeoff + feeders) + conduit &amp; install allowance + data box</t>
   </si>
   <si>
     <t>Switchgear, panels &amp; transformer (Panel sheet)</t>
@@ -1165,123 +1166,126 @@
     <t>DCFC 120kW</t>
   </si>
   <si>
+    <t>Data/comms box $ (one per site)</t>
+  </si>
+  <si>
+    <t>DCFC 120kW Dual</t>
+  </si>
+  <si>
     <t>ADA van stall $ (flat lot)</t>
   </si>
   <si>
-    <t>DCFC 120kW Dual</t>
+    <t>DCFC 160kW</t>
+  </si>
+  <si>
+    <t>300 kcmil</t>
   </si>
   <si>
     <t>ADA standard stall $ (flat lot)</t>
   </si>
   <si>
-    <t>DCFC 160kW</t>
-  </si>
-  <si>
-    <t>300 kcmil</t>
+    <t>DCFC 160kW Dual</t>
   </si>
   <si>
     <t>ADA ambulatory stall $ (flat lot)</t>
   </si>
   <si>
-    <t>DCFC 160kW Dual</t>
+    <t>DCFC 180kW</t>
   </si>
   <si>
     <t>ADA ramp $</t>
   </si>
   <si>
-    <t>DCFC 180kW</t>
+    <t>DCFC 180kW Dual</t>
   </si>
   <si>
     <t>Concrete $/yd (2500 PSI delivered)</t>
   </si>
   <si>
-    <t>DCFC 180kW Dual</t>
-  </si>
-  <si>
     <t>400 kcmil</t>
   </si>
   <si>
+    <t>DCFC 200kW Dual</t>
+  </si>
+  <si>
     <t>Asphalt stall paving $/SF</t>
   </si>
   <si>
-    <t>DCFC 200kW Dual</t>
+    <t>DCFC 240kW</t>
   </si>
   <si>
     <t>Stall patch-back SF per stall (9x18)</t>
   </si>
   <si>
-    <t>DCFC 240kW</t>
+    <t>DCFC 240kW Dual</t>
   </si>
   <si>
     <t>Bollard installed $/ea</t>
   </si>
   <si>
-    <t>DCFC 240kW Dual</t>
+    <t>DCFC 275kW</t>
+  </si>
+  <si>
+    <t>250 kcmil</t>
   </si>
   <si>
     <t>Bollards per charger</t>
   </si>
   <si>
-    <t>DCFC 275kW</t>
-  </si>
-  <si>
-    <t>250 kcmil</t>
+    <t>DCFC 275kW Dual</t>
   </si>
   <si>
     <t>Bollards at switchgear (4-5)</t>
   </si>
   <si>
-    <t>DCFC 275kW Dual</t>
+    <t>DCFC 300kW</t>
   </si>
   <si>
     <t>Bollards at step-down TX + sub-panel</t>
   </si>
   <si>
-    <t>DCFC 300kW</t>
+    <t>DCFC 300kW Dual</t>
   </si>
   <si>
     <t>Forming consumables $/DCFC (anchors, ells, forms)</t>
   </si>
   <si>
-    <t>DCFC 300kW Dual</t>
+    <t>DCFC 360kW</t>
   </si>
   <si>
     <t>Forming consumables $/L2</t>
   </si>
   <si>
-    <t>DCFC 360kW</t>
+    <t>DCFC 360kW Dual</t>
   </si>
   <si>
     <t>Concrete yd per DCFC pad</t>
   </si>
   <si>
-    <t>DCFC 360kW Dual</t>
+    <t>Install $/u = conduit, terminations &amp; install hardware (engine-calibrated) — wire is priced on the Intake's Wire Runs block. 'Install EMT $/u' is the same allowance with surface EMT conduit (garage installs; strut racks are a separate Estimate line). Hardware $/u are budgetary — swap in CTX/vendor quotes.</t>
   </si>
   <si>
     <t>Concrete yd per L2 pad</t>
   </si>
   <si>
-    <t>Install $/u = conduit, terminations &amp; install hardware (engine-calibrated) — wire is priced on the Intake's Wire Runs block. 'Install EMT $/u' is the same allowance with surface EMT conduit (garage installs; strut racks are a separate Estimate line). Hardware $/u are budgetary — swap in CTX/vendor quotes.</t>
-  </si>
-  <si>
     <t>Concrete yd — switchgear pad</t>
   </si>
   <si>
+    <t>Main switchgear 480V (website catalog)</t>
+  </si>
+  <si>
     <t>Concrete yd — step-down TX + sub-panel pad</t>
   </si>
   <si>
-    <t>Main switchgear 480V (website catalog)</t>
+    <t>Size</t>
+  </si>
+  <si>
+    <t>Price</t>
   </si>
   <si>
     <t>Concrete yd per bollard footing</t>
   </si>
   <si>
-    <t>Size</t>
-  </si>
-  <si>
-    <t>Price</t>
-  </si>
-  <si>
     <t>Utility transformer pad $ (DCFC)</t>
   </si>
   <si>
@@ -1315,10 +1319,10 @@
     <t>Permit issuance base $ (AHJ)</t>
   </si>
   <si>
+    <t>Sub-panel / distribution 208V</t>
+  </si>
+  <si>
     <t>Permit issuance $/charger</t>
-  </si>
-  <si>
-    <t>Sub-panel / distribution 208V</t>
   </si>
   <si>
     <t>Utility application $ (DCFC site)</t>
@@ -3609,7 +3613,7 @@
         <v>3000</v>
       </c>
       <c r="C4" s="34">
-        <v>538</v>
+        <v>288</v>
       </c>
       <c r="D4" t="s">
         <v>315</v>
@@ -3648,7 +3652,7 @@
         <v>317</v>
       </c>
       <c r="P4" s="34">
-        <v>803</v>
+        <v>553</v>
       </c>
       <c r="Q4" t="s">
         <v>36</v>
@@ -3674,7 +3678,7 @@
         <v>3500</v>
       </c>
       <c r="C5" s="34">
-        <v>532</v>
+        <v>282</v>
       </c>
       <c r="D5" t="s">
         <v>315</v>
@@ -3713,7 +3717,7 @@
         <v>317</v>
       </c>
       <c r="P5" s="34">
-        <v>790</v>
+        <v>540</v>
       </c>
       <c r="Q5" t="s">
         <v>319</v>
@@ -3739,7 +3743,7 @@
         <v>4000</v>
       </c>
       <c r="C6" s="34">
-        <v>542</v>
+        <v>292</v>
       </c>
       <c r="D6" t="s">
         <v>315</v>
@@ -3778,7 +3782,7 @@
         <v>317</v>
       </c>
       <c r="P6" s="34">
-        <v>813</v>
+        <v>563</v>
       </c>
       <c r="Q6" t="s">
         <v>320</v>
@@ -3804,7 +3808,7 @@
         <v>5000</v>
       </c>
       <c r="C7" s="34">
-        <v>611</v>
+        <v>361</v>
       </c>
       <c r="D7" t="s">
         <v>315</v>
@@ -3843,7 +3847,7 @@
         <v>317</v>
       </c>
       <c r="P7" s="34">
-        <v>938</v>
+        <v>688</v>
       </c>
       <c r="Q7" t="s">
         <v>323</v>
@@ -3869,7 +3873,7 @@
         <v>7500</v>
       </c>
       <c r="C8" s="34">
-        <v>943</v>
+        <v>693</v>
       </c>
       <c r="D8" t="s">
         <v>315</v>
@@ -3908,7 +3912,7 @@
         <v>317</v>
       </c>
       <c r="P8" s="34">
-        <v>1574</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
@@ -3919,7 +3923,7 @@
         <v>5500</v>
       </c>
       <c r="C9" s="34">
-        <v>693</v>
+        <v>443</v>
       </c>
       <c r="D9" t="s">
         <v>315</v>
@@ -3958,7 +3962,7 @@
         <v>317</v>
       </c>
       <c r="P9" s="34">
-        <v>1092</v>
+        <v>842</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.25">
@@ -3969,7 +3973,7 @@
         <v>6500</v>
       </c>
       <c r="C10" s="34">
-        <v>710</v>
+        <v>460</v>
       </c>
       <c r="D10" t="s">
         <v>315</v>
@@ -4008,7 +4012,7 @@
         <v>317</v>
       </c>
       <c r="P10" s="34">
-        <v>1135</v>
+        <v>885</v>
       </c>
       <c r="Q10" t="s">
         <v>328</v>
@@ -4025,7 +4029,7 @@
         <v>8500</v>
       </c>
       <c r="C11" s="34">
-        <v>862</v>
+        <v>612</v>
       </c>
       <c r="D11" t="s">
         <v>315</v>
@@ -4064,7 +4068,7 @@
         <v>317</v>
       </c>
       <c r="P11" s="34">
-        <v>1400</v>
+        <v>1150</v>
       </c>
       <c r="Q11" t="s">
         <v>330</v>
@@ -4081,7 +4085,7 @@
         <v>32000</v>
       </c>
       <c r="C12" s="34">
-        <v>654</v>
+        <v>404</v>
       </c>
       <c r="D12" t="s">
         <v>332</v>
@@ -4120,7 +4124,7 @@
         <v>317</v>
       </c>
       <c r="P12" s="34">
-        <v>1081</v>
+        <v>831</v>
       </c>
       <c r="Q12" t="s">
         <v>334</v>
@@ -4137,7 +4141,7 @@
         <v>35000</v>
       </c>
       <c r="C13" s="34">
-        <v>654</v>
+        <v>404</v>
       </c>
       <c r="D13" t="s">
         <v>332</v>
@@ -4176,7 +4180,7 @@
         <v>317</v>
       </c>
       <c r="P13" s="34">
-        <v>1081</v>
+        <v>831</v>
       </c>
       <c r="Q13" t="s">
         <v>336</v>
@@ -4193,7 +4197,7 @@
         <v>38000</v>
       </c>
       <c r="C14" s="34">
-        <v>657</v>
+        <v>407</v>
       </c>
       <c r="D14" t="s">
         <v>332</v>
@@ -4232,7 +4236,7 @@
         <v>317</v>
       </c>
       <c r="P14" s="34">
-        <v>1092</v>
+        <v>842</v>
       </c>
       <c r="Q14" t="s">
         <v>338</v>
@@ -4249,7 +4253,7 @@
         <v>42000</v>
       </c>
       <c r="C15" s="34">
-        <v>657</v>
+        <v>407</v>
       </c>
       <c r="D15" t="s">
         <v>332</v>
@@ -4288,7 +4292,7 @@
         <v>317</v>
       </c>
       <c r="P15" s="34">
-        <v>1092</v>
+        <v>842</v>
       </c>
       <c r="Q15" t="s">
         <v>340</v>
@@ -4305,7 +4309,7 @@
         <v>52000</v>
       </c>
       <c r="C16" s="34">
-        <v>768</v>
+        <v>518</v>
       </c>
       <c r="D16" t="s">
         <v>332</v>
@@ -4344,7 +4348,7 @@
         <v>317</v>
       </c>
       <c r="P16" s="34">
-        <v>1236</v>
+        <v>986</v>
       </c>
       <c r="Q16" t="s">
         <v>343</v>
@@ -4361,7 +4365,7 @@
         <v>57000</v>
       </c>
       <c r="C17" s="34">
-        <v>768</v>
+        <v>518</v>
       </c>
       <c r="D17" t="s">
         <v>332</v>
@@ -4400,7 +4404,7 @@
         <v>317</v>
       </c>
       <c r="P17" s="34">
-        <v>1236</v>
+        <v>986</v>
       </c>
       <c r="Q17" t="s">
         <v>345</v>
@@ -4417,7 +4421,7 @@
         <v>60000</v>
       </c>
       <c r="C18" s="34">
-        <v>808</v>
+        <v>558</v>
       </c>
       <c r="D18" t="s">
         <v>332</v>
@@ -4456,13 +4460,13 @@
         <v>317</v>
       </c>
       <c r="P18" s="34">
-        <v>1295</v>
+        <v>1045</v>
       </c>
       <c r="Q18" t="s">
         <v>347</v>
       </c>
       <c r="R18" s="34">
-        <v>6500</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.25">
@@ -4473,7 +4477,7 @@
         <v>66000</v>
       </c>
       <c r="C19" s="34">
-        <v>808</v>
+        <v>558</v>
       </c>
       <c r="D19" t="s">
         <v>332</v>
@@ -4512,13 +4516,13 @@
         <v>317</v>
       </c>
       <c r="P19" s="34">
-        <v>1295</v>
+        <v>1045</v>
       </c>
       <c r="Q19" t="s">
         <v>349</v>
       </c>
       <c r="R19" s="34">
-        <v>4900</v>
+        <v>6500</v>
       </c>
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.25">
@@ -4529,7 +4533,7 @@
         <v>72000</v>
       </c>
       <c r="C20" s="34">
-        <v>1003</v>
+        <v>753</v>
       </c>
       <c r="D20" t="s">
         <v>332</v>
@@ -4568,13 +4572,13 @@
         <v>317</v>
       </c>
       <c r="P20" s="34">
-        <v>1670</v>
+        <v>1420</v>
       </c>
       <c r="Q20" t="s">
         <v>352</v>
       </c>
       <c r="R20" s="34">
-        <v>3500</v>
+        <v>4900</v>
       </c>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.25">
@@ -4585,7 +4589,7 @@
         <v>79000</v>
       </c>
       <c r="C21" s="34">
-        <v>1003</v>
+        <v>753</v>
       </c>
       <c r="D21" t="s">
         <v>332</v>
@@ -4624,13 +4628,13 @@
         <v>317</v>
       </c>
       <c r="P21" s="34">
-        <v>1670</v>
+        <v>1420</v>
       </c>
       <c r="Q21" t="s">
         <v>354</v>
       </c>
       <c r="R21" s="34">
-        <v>5200</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.25">
@@ -4641,7 +4645,7 @@
         <v>80000</v>
       </c>
       <c r="C22" s="34">
-        <v>1086</v>
+        <v>836</v>
       </c>
       <c r="D22" t="s">
         <v>332</v>
@@ -4680,13 +4684,13 @@
         <v>317</v>
       </c>
       <c r="P22" s="34">
-        <v>1780</v>
+        <v>1530</v>
       </c>
       <c r="Q22" t="s">
         <v>356</v>
       </c>
       <c r="R22" s="34">
-        <v>165</v>
+        <v>5200</v>
       </c>
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.25">
@@ -4697,7 +4701,7 @@
         <v>88000</v>
       </c>
       <c r="C23" s="34">
-        <v>1086</v>
+        <v>836</v>
       </c>
       <c r="D23" t="s">
         <v>332</v>
@@ -4736,13 +4740,13 @@
         <v>317</v>
       </c>
       <c r="P23" s="34">
-        <v>1780</v>
+        <v>1530</v>
       </c>
       <c r="Q23" t="s">
-        <v>213</v>
+        <v>358</v>
       </c>
       <c r="R23" s="34">
-        <v>125</v>
+        <v>165</v>
       </c>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.25">
@@ -4753,7 +4757,7 @@
         <v>92000</v>
       </c>
       <c r="C24" s="34">
-        <v>1182</v>
+        <v>932</v>
       </c>
       <c r="D24" t="s">
         <v>332</v>
@@ -4786,19 +4790,19 @@
         <v>3</v>
       </c>
       <c r="N24" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="O24" t="s">
         <v>317</v>
       </c>
       <c r="P24" s="34">
-        <v>2024</v>
+        <v>1774</v>
       </c>
       <c r="Q24" t="s">
-        <v>359</v>
+        <v>213</v>
       </c>
       <c r="R24" s="34">
-        <v>5</v>
+        <v>125</v>
       </c>
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.25">
@@ -4809,7 +4813,7 @@
         <v>100000</v>
       </c>
       <c r="C25" s="34">
-        <v>1182</v>
+        <v>932</v>
       </c>
       <c r="D25" t="s">
         <v>332</v>
@@ -4842,19 +4846,19 @@
         <v>3</v>
       </c>
       <c r="N25" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="O25" t="s">
         <v>317</v>
       </c>
       <c r="P25" s="34">
-        <v>2024</v>
+        <v>1774</v>
       </c>
       <c r="Q25" t="s">
         <v>361</v>
       </c>
-      <c r="R25" s="8">
-        <v>162</v>
+      <c r="R25" s="34">
+        <v>5</v>
       </c>
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.25">
@@ -4865,7 +4869,7 @@
         <v>105000</v>
       </c>
       <c r="C26" s="34">
-        <v>1518</v>
+        <v>1268</v>
       </c>
       <c r="D26" t="s">
         <v>332</v>
@@ -4904,13 +4908,13 @@
         <v>317</v>
       </c>
       <c r="P26" s="34">
-        <v>2374</v>
+        <v>2124</v>
       </c>
       <c r="Q26" t="s">
         <v>363</v>
       </c>
-      <c r="R26" s="34">
-        <v>110</v>
+      <c r="R26" s="8">
+        <v>162</v>
       </c>
     </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.25">
@@ -4921,7 +4925,7 @@
         <v>115000</v>
       </c>
       <c r="C27" s="34">
-        <v>1518</v>
+        <v>1268</v>
       </c>
       <c r="D27" t="s">
         <v>332</v>
@@ -4960,13 +4964,13 @@
         <v>317</v>
       </c>
       <c r="P27" s="34">
-        <v>2374</v>
+        <v>2124</v>
       </c>
       <c r="Q27" t="s">
         <v>365</v>
       </c>
-      <c r="R27" s="8">
-        <v>2</v>
+      <c r="R27" s="34">
+        <v>110</v>
       </c>
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.25">
@@ -4977,7 +4981,7 @@
         <v>120000</v>
       </c>
       <c r="C28" s="34">
-        <v>1816</v>
+        <v>1566</v>
       </c>
       <c r="D28" t="s">
         <v>332</v>
@@ -5016,13 +5020,13 @@
         <v>317</v>
       </c>
       <c r="P28" s="34">
-        <v>3043</v>
+        <v>2793</v>
       </c>
       <c r="Q28" t="s">
         <v>368</v>
       </c>
       <c r="R28" s="8">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.25">
@@ -5033,7 +5037,7 @@
         <v>130000</v>
       </c>
       <c r="C29" s="34">
-        <v>1816</v>
+        <v>1566</v>
       </c>
       <c r="D29" t="s">
         <v>332</v>
@@ -5072,13 +5076,13 @@
         <v>317</v>
       </c>
       <c r="P29" s="34">
-        <v>3043</v>
+        <v>2793</v>
       </c>
       <c r="Q29" t="s">
         <v>370</v>
       </c>
       <c r="R29" s="8">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.25">
@@ -5089,7 +5093,7 @@
         <v>135000</v>
       </c>
       <c r="C30" s="34">
-        <v>1816</v>
+        <v>1566</v>
       </c>
       <c r="D30" t="s">
         <v>332</v>
@@ -5128,13 +5132,13 @@
         <v>317</v>
       </c>
       <c r="P30" s="34">
-        <v>3043</v>
+        <v>2793</v>
       </c>
       <c r="Q30" t="s">
         <v>372</v>
       </c>
-      <c r="R30" s="34">
-        <v>550</v>
+      <c r="R30" s="8">
+        <v>3</v>
       </c>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.25">
@@ -5145,7 +5149,7 @@
         <v>147000</v>
       </c>
       <c r="C31" s="34">
-        <v>1816</v>
+        <v>1566</v>
       </c>
       <c r="D31" t="s">
         <v>332</v>
@@ -5184,13 +5188,13 @@
         <v>317</v>
       </c>
       <c r="P31" s="34">
-        <v>3043</v>
+        <v>2793</v>
       </c>
       <c r="Q31" t="s">
         <v>374</v>
       </c>
       <c r="R31" s="34">
-        <v>275</v>
+        <v>550</v>
       </c>
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.25">
@@ -5201,7 +5205,7 @@
         <v>155000</v>
       </c>
       <c r="C32" s="34">
-        <v>2007</v>
+        <v>1757</v>
       </c>
       <c r="D32" t="s">
         <v>332</v>
@@ -5240,13 +5244,13 @@
         <v>317</v>
       </c>
       <c r="P32" s="34">
-        <v>3483</v>
+        <v>3233</v>
       </c>
       <c r="Q32" t="s">
         <v>376</v>
       </c>
-      <c r="R32" s="8">
-        <v>0.75</v>
+      <c r="R32" s="34">
+        <v>275</v>
       </c>
     </row>
     <row r="33" spans="1:18" x14ac:dyDescent="0.25">
@@ -5257,7 +5261,7 @@
         <v>168000</v>
       </c>
       <c r="C33" s="34">
-        <v>2007</v>
+        <v>1757</v>
       </c>
       <c r="D33" t="s">
         <v>332</v>
@@ -5296,13 +5300,13 @@
         <v>317</v>
       </c>
       <c r="P33" s="34">
-        <v>3483</v>
+        <v>3233</v>
       </c>
       <c r="Q33" t="s">
         <v>378</v>
       </c>
       <c r="R33" s="8">
-        <v>0.35</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="34" spans="1:18" x14ac:dyDescent="0.25">
@@ -5313,7 +5317,7 @@
         <v>380</v>
       </c>
       <c r="R34" s="8">
-        <v>1.75</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="35" spans="17:18" x14ac:dyDescent="0.25">
@@ -5321,7 +5325,7 @@
         <v>381</v>
       </c>
       <c r="R35" s="8">
-        <v>0.5</v>
+        <v>1.75</v>
       </c>
     </row>
     <row r="36" spans="1:18" x14ac:dyDescent="0.25">
@@ -5332,7 +5336,7 @@
         <v>383</v>
       </c>
       <c r="R36" s="8">
-        <v>0.08</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="37" spans="1:18" x14ac:dyDescent="0.25">
@@ -5345,8 +5349,8 @@
       <c r="Q37" t="s">
         <v>386</v>
       </c>
-      <c r="R37" s="34">
-        <v>5000</v>
+      <c r="R37" s="8">
+        <v>0.08</v>
       </c>
     </row>
     <row r="38" spans="1:18" x14ac:dyDescent="0.25">
@@ -5360,7 +5364,7 @@
         <v>387</v>
       </c>
       <c r="R38" s="34">
-        <v>1500</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="39" spans="1:18" x14ac:dyDescent="0.25">
@@ -5374,7 +5378,7 @@
         <v>388</v>
       </c>
       <c r="R39" s="34">
-        <v>250</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="40" spans="1:18" x14ac:dyDescent="0.25">
@@ -5388,7 +5392,7 @@
         <v>389</v>
       </c>
       <c r="R40" s="34">
-        <v>3519</v>
+        <v>250</v>
       </c>
     </row>
     <row r="41" spans="1:18" x14ac:dyDescent="0.25">
@@ -5402,7 +5406,7 @@
         <v>390</v>
       </c>
       <c r="R41" s="34">
-        <v>261</v>
+        <v>3519</v>
       </c>
     </row>
     <row r="42" spans="1:18" x14ac:dyDescent="0.25">
@@ -5416,7 +5420,7 @@
         <v>391</v>
       </c>
       <c r="R42" s="34">
-        <v>4043</v>
+        <v>261</v>
       </c>
     </row>
     <row r="43" spans="1:18" x14ac:dyDescent="0.25">
@@ -5430,7 +5434,7 @@
         <v>392</v>
       </c>
       <c r="R43" s="34">
-        <v>35</v>
+        <v>4043</v>
       </c>
     </row>
     <row r="44" spans="1:18" x14ac:dyDescent="0.25">
@@ -5444,7 +5448,7 @@
         <v>393</v>
       </c>
       <c r="R44" s="34">
-        <v>28</v>
+        <v>35</v>
       </c>
     </row>
     <row r="45" spans="1:18" x14ac:dyDescent="0.25">
@@ -5458,7 +5462,7 @@
         <v>394</v>
       </c>
       <c r="R45" s="34">
-        <v>3.25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="46" spans="1:18" x14ac:dyDescent="0.25">
@@ -5471,8 +5475,8 @@
       <c r="Q46" t="s">
         <v>395</v>
       </c>
-      <c r="R46" s="8">
-        <v>100</v>
+      <c r="R46" s="34">
+        <v>3.25</v>
       </c>
     </row>
     <row r="47" spans="1:18" x14ac:dyDescent="0.25">
@@ -5485,8 +5489,8 @@
       <c r="Q47" t="s">
         <v>396</v>
       </c>
-      <c r="R47" s="34">
-        <v>200</v>
+      <c r="R47" s="8">
+        <v>100</v>
       </c>
     </row>
     <row r="48" spans="17:18" x14ac:dyDescent="0.25">
@@ -5494,7 +5498,7 @@
         <v>397</v>
       </c>
       <c r="R48" s="34">
-        <v>60</v>
+        <v>200</v>
       </c>
     </row>
     <row r="49" spans="1:18" x14ac:dyDescent="0.25">
@@ -5505,7 +5509,7 @@
         <v>399</v>
       </c>
       <c r="R49" s="34">
-        <v>2500</v>
+        <v>60</v>
       </c>
     </row>
     <row r="50" spans="1:18" x14ac:dyDescent="0.25">
@@ -5519,15 +5523,21 @@
         <v>400</v>
       </c>
       <c r="R50" s="34">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="51" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>150</v>
       </c>
       <c r="B51" s="34">
         <v>1000</v>
+      </c>
+      <c r="Q51" t="s">
+        <v>401</v>
+      </c>
+      <c r="R51" s="34">
+        <v>800</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
@@ -5572,7 +5582,7 @@
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
@@ -5641,7 +5651,7 @@
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" s="3" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.25">
@@ -5750,7 +5760,7 @@
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A83" s="3" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.25">
@@ -5787,7 +5797,7 @@
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A89" s="3" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.25">
@@ -5972,7 +5982,7 @@
     </row>
     <row r="127" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A127" s="3" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
     </row>
     <row r="128" spans="1:5" x14ac:dyDescent="0.25">
@@ -5980,21 +5990,21 @@
         <v>384</v>
       </c>
       <c r="B128" s="7" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="C128" s="7" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="D128" s="7" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="E128" s="7" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B129" s="34">
         <v>0</v>
@@ -6011,7 +6021,7 @@
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="B130" s="34">
         <v>0</v>
@@ -6028,7 +6038,7 @@
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="B131" s="34">
         <v>0.30329</v>
@@ -6045,7 +6055,7 @@
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="B132" s="34">
         <v>0.56613</v>
@@ -6079,7 +6089,7 @@
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="B134" s="34">
         <v>1.33293</v>
@@ -6113,7 +6123,7 @@
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="B136" s="34">
         <v>2.1044</v>
@@ -6164,7 +6174,7 @@
     </row>
     <row r="139" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="B139" s="34">
         <v>3.63758</v>
@@ -6266,7 +6276,7 @@
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B145" s="34">
         <v>10.60671</v>
@@ -6283,7 +6293,7 @@
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="B146" s="34">
         <v>11.334</v>
@@ -6300,7 +6310,7 @@
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="B147" s="34">
         <v>13.30059</v>
@@ -6334,7 +6344,7 @@
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="B149" s="34">
         <v>0</v>
@@ -6351,7 +6361,7 @@
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B150" s="34">
         <v>25.921</v>
@@ -6368,7 +6378,7 @@
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="B151" s="34">
         <v>0</v>
@@ -6385,7 +6395,7 @@
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="B152" s="34">
         <v>0</v>
@@ -6402,7 +6412,7 @@
     </row>
     <row r="153" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="B153" s="34">
         <v>34.398</v>
@@ -6419,7 +6429,7 @@
     </row>
     <row r="154" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A154" s="2" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
     </row>
   </sheetData>
@@ -6438,142 +6448,142 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="19" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="64" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="64" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="64" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="64" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="64" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="64" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="64" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="64" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="64" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="64" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="64" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="64" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="64" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" s="64" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" s="64" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="64" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="64" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" s="64" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" s="64" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" s="64" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" s="64" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" s="64" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="64" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" s="64" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" s="64" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" s="64" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" s="64" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
@@ -6583,22 +6593,22 @@
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" s="19" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" s="64" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" s="64" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" s="64" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
@@ -6608,17 +6618,17 @@
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" s="19" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" s="64" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" s="64" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
@@ -6628,57 +6638,57 @@
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" s="19" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" s="64" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" s="64" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" s="64" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" s="64" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" s="64" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" s="64" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" s="64" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" s="64" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" s="64" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" s="64" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
     </row>
   </sheetData>
@@ -12511,7 +12521,7 @@
         <v>171</v>
       </c>
       <c r="B7" s="9">
-        <f>WireTotal+SUM(Intake!E23:E34)</f>
+        <f>WireTotal+SUM(Intake!E23:E34)+IF(NTotal&gt;0,DataBoxCost,0)</f>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -13152,7 +13162,7 @@
         <v>1</v>
       </c>
       <c r="D3" s="42">
-        <f>Estimate!B7+Estimate!B10</f>
+        <f>Estimate!B7+Estimate!B10+Estimate!B15</f>
       </c>
       <c r="E3" s="43">
         <f>ContingencyPct</f>
@@ -13360,7 +13370,7 @@
         <v>1</v>
       </c>
       <c r="D12" s="42">
-        <f>Estimate!B18+Estimate!B15</f>
+        <f>Estimate!B18</f>
       </c>
       <c r="E12" s="43">
         <f>ContingencyPct</f>

</xml_diff>

<commit_message>
Switchgear ladder: add 600A and 3200A, re-set 3000/4000/5000A on Larson's published boards
GEAR_CATALOG "Main switchgear" 480V: 600A $25,500 (new), 3000A $58,842
(Larson main-only Type 3R, was $65,000), 3200A $62,200 (new, $16.76/A
slope), 4000A $75,600 (was $67,500), 5000A $100,000 (was $70,000). 400A to
2500A unchanged. Both new frames join SWITCHGEAR_480V_A and
STANDARD_BREAKERS_A so the panel schedule can pick them; the standalone
template regenerates its SgSizes/SgTable from the catalog (verify pin now
3000A = $58,842); the refdata parity test records 3000/4000/5000A as
deliberate departures from the intake's RefData table.

Basis: Larson Electronics publishes prices — the user's $59,593 "3200A"
quote is their switch-only 2 IN 2 OUT NEMA 12 metal-enclosed gear; their
800A and 3000A main-only boards ($21,968 / $58,842) give the main-breaker
slope used here. Research on file in memory (larson-switchgear-prices).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/RFC-Template.xlsx
+++ b/templates/RFC-Template.xlsx
@@ -19,19 +19,19 @@
   </sheets>
   <definedNames>
     <definedName name="ModelTable">RateCard!$A$4:$P$38</definedName>
-    <definedName name="SgSizes">RateCard!$A$43:$A$52</definedName>
-    <definedName name="SgTable">RateCard!$A$43:$B$52</definedName>
-    <definedName name="PnlSizes">RateCard!$A$56:$A$61</definedName>
-    <definedName name="PnlTable">RateCard!$A$56:$B$61</definedName>
-    <definedName name="TxSizes">RateCard!$A$65:$A$71</definedName>
-    <definedName name="TxTable">RateCard!$A$65:$B$71</definedName>
-    <definedName name="Brk480Sizes">RateCard!$A$75:$A$86</definedName>
-    <definedName name="BrkTbl480">RateCard!$A$75:$B$86</definedName>
-    <definedName name="Brk208Sizes">RateCard!$A$90:$A$92</definedName>
-    <definedName name="BrkTbl208">RateCard!$A$90:$B$92</definedName>
-    <definedName name="StdBrk">RateCard!$A$95:$A$130</definedName>
-    <definedName name="WireSizes">RateCard!$A$134:$A$158</definedName>
-    <definedName name="WireTable">RateCard!$A$134:$E$158</definedName>
+    <definedName name="SgSizes">RateCard!$A$43:$A$54</definedName>
+    <definedName name="SgTable">RateCard!$A$43:$B$54</definedName>
+    <definedName name="PnlSizes">RateCard!$A$58:$A$63</definedName>
+    <definedName name="PnlTable">RateCard!$A$58:$B$63</definedName>
+    <definedName name="TxSizes">RateCard!$A$67:$A$73</definedName>
+    <definedName name="TxTable">RateCard!$A$67:$B$73</definedName>
+    <definedName name="Brk480Sizes">RateCard!$A$77:$A$88</definedName>
+    <definedName name="BrkTbl480">RateCard!$A$77:$B$88</definedName>
+    <definedName name="Brk208Sizes">RateCard!$A$92:$A$94</definedName>
+    <definedName name="BrkTbl208">RateCard!$A$92:$B$94</definedName>
+    <definedName name="StdBrk">RateCard!$A$97:$A$133</definedName>
+    <definedName name="WireSizes">RateCard!$A$137:$A$161</definedName>
+    <definedName name="WireTable">RateCard!$A$137:$E$161</definedName>
     <definedName name="TerrainTable">RateCard!$Q$4:$U$7</definedName>
     <definedName name="TrenchRate">RateCard!$R$10</definedName>
     <definedName name="ContingencyPct">RateCard!$R$11</definedName>
@@ -3359,7 +3359,7 @@
       <formula1>"Trenched,Surface EMT,Hybrid"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B53:B67">
-      <formula1>RateCard!$A$134:$A$158</formula1>
+      <formula1>RateCard!$A$137:$A$161</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="B78:B83">
       <formula1>"Yes,No"</formula1>
@@ -3530,7 +3530,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:U159"/>
+  <dimension ref="A1:U162"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -4099,7 +4099,7 @@
         <v>23600</v>
       </c>
       <c r="C12" s="33">
-        <v>404</v>
+        <v>399</v>
       </c>
       <c r="D12" t="s">
         <v>332</v>
@@ -4138,7 +4138,7 @@
         <v>317</v>
       </c>
       <c r="P12" s="33">
-        <v>831</v>
+        <v>827</v>
       </c>
       <c r="Q12" t="s">
         <v>334</v>
@@ -4155,7 +4155,7 @@
         <v>23600</v>
       </c>
       <c r="C13" s="33">
-        <v>404</v>
+        <v>399</v>
       </c>
       <c r="D13" t="s">
         <v>332</v>
@@ -4194,7 +4194,7 @@
         <v>317</v>
       </c>
       <c r="P13" s="33">
-        <v>831</v>
+        <v>827</v>
       </c>
       <c r="Q13" t="s">
         <v>336</v>
@@ -4211,7 +4211,7 @@
         <v>28500</v>
       </c>
       <c r="C14" s="33">
-        <v>407</v>
+        <v>402</v>
       </c>
       <c r="D14" t="s">
         <v>332</v>
@@ -4250,7 +4250,7 @@
         <v>317</v>
       </c>
       <c r="P14" s="33">
-        <v>842</v>
+        <v>837</v>
       </c>
       <c r="Q14" t="s">
         <v>338</v>
@@ -4267,7 +4267,7 @@
         <v>28500</v>
       </c>
       <c r="C15" s="33">
-        <v>407</v>
+        <v>402</v>
       </c>
       <c r="D15" t="s">
         <v>332</v>
@@ -4306,7 +4306,7 @@
         <v>317</v>
       </c>
       <c r="P15" s="33">
-        <v>842</v>
+        <v>837</v>
       </c>
       <c r="Q15" t="s">
         <v>340</v>
@@ -5663,10 +5663,10 @@
     </row>
     <row r="44" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A44">
-        <v>800</v>
+        <v>600</v>
       </c>
       <c r="B44" s="33">
-        <v>31187</v>
+        <v>25500</v>
       </c>
       <c r="Q44" t="s">
         <v>399</v>
@@ -5677,10 +5677,10 @@
     </row>
     <row r="45" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A45">
-        <v>1000</v>
+        <v>800</v>
       </c>
       <c r="B45" s="33">
-        <v>36812.5</v>
+        <v>31187</v>
       </c>
       <c r="Q45" t="s">
         <v>400</v>
@@ -5691,10 +5691,10 @@
     </row>
     <row r="46" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A46">
-        <v>1200</v>
+        <v>1000</v>
       </c>
       <c r="B46" s="33">
-        <v>43292.68</v>
+        <v>36812.5</v>
       </c>
       <c r="Q46" t="s">
         <v>401</v>
@@ -5705,10 +5705,10 @@
     </row>
     <row r="47" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A47">
-        <v>1600</v>
+        <v>1200</v>
       </c>
       <c r="B47" s="33">
-        <v>56750</v>
+        <v>43292.68</v>
       </c>
       <c r="Q47" t="s">
         <v>402</v>
@@ -5719,10 +5719,10 @@
     </row>
     <row r="48" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A48">
-        <v>2000</v>
+        <v>1600</v>
       </c>
       <c r="B48" s="33">
-        <v>55000</v>
+        <v>56750</v>
       </c>
       <c r="Q48" t="s">
         <v>403</v>
@@ -5733,10 +5733,10 @@
     </row>
     <row r="49" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A49">
-        <v>2500</v>
+        <v>2000</v>
       </c>
       <c r="B49" s="33">
-        <v>60000</v>
+        <v>55000</v>
       </c>
       <c r="Q49" t="s">
         <v>404</v>
@@ -5747,10 +5747,10 @@
     </row>
     <row r="50" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A50">
-        <v>3000</v>
+        <v>2500</v>
       </c>
       <c r="B50" s="33">
-        <v>65000</v>
+        <v>60000</v>
       </c>
       <c r="Q50" t="s">
         <v>405</v>
@@ -5761,10 +5761,10 @@
     </row>
     <row r="51" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A51">
-        <v>4000</v>
+        <v>3000</v>
       </c>
       <c r="B51" s="33">
-        <v>67500</v>
+        <v>58842</v>
       </c>
       <c r="Q51" t="s">
         <v>406</v>
@@ -5775,922 +5775,943 @@
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52">
+        <v>3200</v>
+      </c>
+      <c r="B52" s="33">
+        <v>62200</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <v>4000</v>
+      </c>
+      <c r="B53" s="33">
+        <v>75600</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A54">
         <v>5000</v>
       </c>
-      <c r="B52" s="33">
-        <v>70000</v>
-      </c>
-    </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A54" s="3" t="s">
+      <c r="B54" s="33">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A56" s="3" t="s">
         <v>407</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A55" s="7" t="s">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A57" s="7" t="s">
         <v>395</v>
       </c>
-      <c r="B55" s="7" t="s">
+      <c r="B57" s="7" t="s">
         <v>396</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A56">
-        <v>150</v>
-      </c>
-      <c r="B56" s="33">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A57">
-        <v>250</v>
-      </c>
-      <c r="B57" s="33">
-        <v>1120</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58">
-        <v>400</v>
+        <v>150</v>
       </c>
       <c r="B58" s="33">
-        <v>1660</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59">
-        <v>600</v>
+        <v>250</v>
       </c>
       <c r="B59" s="33">
-        <v>5387</v>
+        <v>1120</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60">
-        <v>800</v>
+        <v>400</v>
       </c>
       <c r="B60" s="33">
-        <v>4650</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61">
+        <v>600</v>
+      </c>
+      <c r="B61" s="33">
+        <v>5387</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62">
+        <v>800</v>
+      </c>
+      <c r="B62" s="33">
+        <v>4650</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A63">
         <v>1000</v>
       </c>
-      <c r="B61" s="33">
+      <c r="B63" s="33">
         <v>30000</v>
       </c>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A63" s="3" t="s">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A65" s="3" t="s">
         <v>408</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A64" s="7" t="s">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A66" s="7" t="s">
         <v>395</v>
       </c>
-      <c r="B64" s="7" t="s">
+      <c r="B66" s="7" t="s">
         <v>396</v>
-      </c>
-    </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A65">
-        <v>75</v>
-      </c>
-      <c r="B65" s="33">
-        <v>2970</v>
-      </c>
-    </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A66">
-        <v>112.5</v>
-      </c>
-      <c r="B66" s="33">
-        <v>3250</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67">
-        <v>150</v>
+        <v>75</v>
       </c>
       <c r="B67" s="33">
-        <v>5298</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68">
-        <v>175</v>
+        <v>112.5</v>
       </c>
       <c r="B68" s="33">
-        <v>6000</v>
+        <v>3250</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69">
-        <v>225</v>
+        <v>150</v>
       </c>
       <c r="B69" s="33">
-        <v>7144</v>
+        <v>5298</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70">
-        <v>300</v>
+        <v>175</v>
       </c>
       <c r="B70" s="33">
-        <v>10493</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71">
+        <v>225</v>
+      </c>
+      <c r="B71" s="33">
+        <v>7144</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A72">
+        <v>300</v>
+      </c>
+      <c r="B72" s="33">
+        <v>10493</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A73">
         <v>500</v>
       </c>
-      <c r="B71" s="33">
+      <c r="B73" s="33">
         <v>14500</v>
       </c>
     </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A73" s="3" t="s">
+    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A75" s="3" t="s">
         <v>409</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A74" s="7" t="s">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A76" s="7" t="s">
         <v>395</v>
       </c>
-      <c r="B74" s="7" t="s">
+      <c r="B76" s="7" t="s">
         <v>396</v>
-      </c>
-    </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A75">
-        <v>100</v>
-      </c>
-      <c r="B75" s="33">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A76">
-        <v>125</v>
-      </c>
-      <c r="B76" s="33">
-        <v>420</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="B77" s="33">
-        <v>480</v>
+        <v>350</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78">
-        <v>175</v>
+        <v>125</v>
       </c>
       <c r="B78" s="33">
-        <v>550</v>
+        <v>420</v>
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="B79" s="33">
-        <v>650</v>
+        <v>480</v>
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80">
-        <v>225</v>
+        <v>175</v>
       </c>
       <c r="B80" s="33">
-        <v>700</v>
+        <v>550</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="B81" s="33">
-        <v>750</v>
+        <v>650</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82">
-        <v>300</v>
+        <v>225</v>
       </c>
       <c r="B82" s="33">
-        <v>800</v>
+        <v>700</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83">
-        <v>350</v>
+        <v>250</v>
       </c>
       <c r="B83" s="33">
-        <v>1000</v>
+        <v>750</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="B84" s="33">
-        <v>1200</v>
+        <v>800</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85">
-        <v>500</v>
+        <v>350</v>
       </c>
       <c r="B85" s="33">
-        <v>1800</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86">
+        <v>400</v>
+      </c>
+      <c r="B86" s="33">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A87">
+        <v>500</v>
+      </c>
+      <c r="B87" s="33">
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A88">
         <v>600</v>
       </c>
-      <c r="B86" s="33">
+      <c r="B88" s="33">
         <v>2200</v>
       </c>
     </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A88" s="3" t="s">
+    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A90" s="3" t="s">
         <v>410</v>
       </c>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A89" s="7" t="s">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A91" s="7" t="s">
         <v>395</v>
       </c>
-      <c r="B89" s="7" t="s">
+      <c r="B91" s="7" t="s">
         <v>396</v>
-      </c>
-    </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A90">
-        <v>40</v>
-      </c>
-      <c r="B90" s="33">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A91">
-        <v>50</v>
-      </c>
-      <c r="B91" s="33">
-        <v>75</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92">
+        <v>40</v>
+      </c>
+      <c r="B92" s="33">
         <v>60</v>
       </c>
-      <c r="B92" s="33">
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A93">
+        <v>50</v>
+      </c>
+      <c r="B93" s="33">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A94">
+        <v>60</v>
+      </c>
+      <c r="B94" s="33">
         <v>90</v>
       </c>
     </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A94" s="3" t="s">
+    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A96" s="3" t="s">
         <v>411</v>
-      </c>
-    </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A95">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A96">
-        <v>20</v>
       </c>
     </row>
     <row r="97" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A97">
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="98" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A98">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="99" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A99">
-        <v>35</v>
+        <v>25</v>
       </c>
     </row>
     <row r="100" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A100">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="101" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A101">
-        <v>45</v>
+        <v>35</v>
       </c>
     </row>
     <row r="102" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A102">
-        <v>50</v>
+        <v>40</v>
       </c>
     </row>
     <row r="103" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A103">
-        <v>60</v>
+        <v>45</v>
       </c>
     </row>
     <row r="104" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A104">
-        <v>70</v>
+        <v>50</v>
       </c>
     </row>
     <row r="105" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A105">
-        <v>80</v>
+        <v>60</v>
       </c>
     </row>
     <row r="106" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A106">
-        <v>90</v>
+        <v>70</v>
       </c>
     </row>
     <row r="107" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A107">
-        <v>100</v>
+        <v>80</v>
       </c>
     </row>
     <row r="108" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A108">
-        <v>110</v>
+        <v>90</v>
       </c>
     </row>
     <row r="109" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A109">
-        <v>125</v>
+        <v>100</v>
       </c>
     </row>
     <row r="110" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A110">
-        <v>150</v>
+        <v>110</v>
       </c>
     </row>
     <row r="111" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A111">
-        <v>175</v>
+        <v>125</v>
       </c>
     </row>
     <row r="112" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A112">
-        <v>200</v>
+        <v>150</v>
       </c>
     </row>
     <row r="113" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A113">
-        <v>225</v>
+        <v>175</v>
       </c>
     </row>
     <row r="114" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A114">
-        <v>250</v>
+        <v>200</v>
       </c>
     </row>
     <row r="115" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A115">
-        <v>300</v>
+        <v>225</v>
       </c>
     </row>
     <row r="116" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A116">
-        <v>350</v>
+        <v>250</v>
       </c>
     </row>
     <row r="117" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A117">
-        <v>400</v>
+        <v>300</v>
       </c>
     </row>
     <row r="118" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A118">
-        <v>450</v>
+        <v>350</v>
       </c>
     </row>
     <row r="119" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A119">
-        <v>500</v>
+        <v>400</v>
       </c>
     </row>
     <row r="120" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A120">
-        <v>600</v>
+        <v>450</v>
       </c>
     </row>
     <row r="121" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A121">
-        <v>700</v>
+        <v>500</v>
       </c>
     </row>
     <row r="122" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A122">
-        <v>800</v>
+        <v>600</v>
       </c>
     </row>
     <row r="123" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A123">
-        <v>1000</v>
+        <v>700</v>
       </c>
     </row>
     <row r="124" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A124">
-        <v>1200</v>
+        <v>800</v>
       </c>
     </row>
     <row r="125" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A125">
-        <v>1600</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="126" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A126">
-        <v>2000</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="127" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A127">
-        <v>2500</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="128" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A128">
-        <v>3000</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="129" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A129">
-        <v>4000</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="130" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A130">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="131" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A131">
+        <v>3200</v>
+      </c>
+    </row>
+    <row r="132" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A132">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="133" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A133">
         <v>5000</v>
       </c>
     </row>
-    <row r="132" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A132" s="3" t="s">
+    <row r="135" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A135" s="3" t="s">
         <v>412</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A133" s="7" t="s">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A136" s="7" t="s">
         <v>395</v>
       </c>
-      <c r="B133" s="7" t="s">
+      <c r="B136" s="7" t="s">
         <v>413</v>
       </c>
-      <c r="C133" s="7" t="s">
+      <c r="C136" s="7" t="s">
         <v>414</v>
       </c>
-      <c r="D133" s="7" t="s">
+      <c r="D136" s="7" t="s">
         <v>415</v>
       </c>
-      <c r="E133" s="7" t="s">
+      <c r="E136" s="7" t="s">
         <v>416</v>
-      </c>
-    </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A134" t="s">
-        <v>417</v>
-      </c>
-      <c r="B134" s="33">
-        <v>0</v>
-      </c>
-      <c r="C134" s="33">
-        <v>0</v>
-      </c>
-      <c r="D134">
-        <v>20</v>
-      </c>
-      <c r="E134">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A135" t="s">
-        <v>418</v>
-      </c>
-      <c r="B135" s="33">
-        <v>0</v>
-      </c>
-      <c r="C135" s="33">
-        <v>0</v>
-      </c>
-      <c r="D135">
-        <v>25</v>
-      </c>
-      <c r="E135">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A136" t="s">
-        <v>419</v>
-      </c>
-      <c r="B136" s="33">
-        <v>0.30329</v>
-      </c>
-      <c r="C136" s="33">
-        <v>0.28</v>
-      </c>
-      <c r="D136">
-        <v>35</v>
-      </c>
-      <c r="E136">
-        <v>30</v>
       </c>
     </row>
     <row r="137" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>380</v>
+        <v>417</v>
       </c>
       <c r="B137" s="33">
-        <v>0.56613</v>
+        <v>0</v>
       </c>
       <c r="C137" s="33">
         <v>0</v>
       </c>
       <c r="D137">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="E137">
-        <v>40</v>
+        <v>15</v>
       </c>
     </row>
     <row r="138" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>316</v>
+        <v>418</v>
       </c>
       <c r="B138" s="33">
-        <v>0.87104</v>
+        <v>0</v>
       </c>
       <c r="C138" s="33">
-        <v>0.30636</v>
+        <v>0</v>
       </c>
       <c r="D138">
-        <v>65</v>
+        <v>25</v>
       </c>
       <c r="E138">
-        <v>50</v>
+        <v>20</v>
       </c>
     </row>
     <row r="139" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="B139" s="33">
-        <v>1.33293</v>
+        <v>0.30329</v>
       </c>
       <c r="C139" s="33">
-        <v>0.37998</v>
+        <v>0.28</v>
       </c>
       <c r="D139">
-        <v>85</v>
+        <v>35</v>
       </c>
       <c r="E139">
-        <v>65</v>
+        <v>30</v>
       </c>
     </row>
     <row r="140" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>322</v>
+        <v>380</v>
       </c>
       <c r="B140" s="33">
-        <v>1.68126</v>
+        <v>0.56613</v>
       </c>
       <c r="C140" s="33">
-        <v>0.36681</v>
+        <v>0</v>
       </c>
       <c r="D140">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="E140">
-        <v>75</v>
+        <v>40</v>
       </c>
     </row>
     <row r="141" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>421</v>
+        <v>316</v>
       </c>
       <c r="B141" s="33">
-        <v>2.1044</v>
+        <v>0.87104</v>
       </c>
       <c r="C141" s="33">
-        <v>0.4821</v>
+        <v>0.30636</v>
       </c>
       <c r="D141">
-        <v>115</v>
+        <v>65</v>
       </c>
       <c r="E141">
-        <v>90</v>
+        <v>50</v>
       </c>
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>325</v>
+        <v>420</v>
       </c>
       <c r="B142" s="33">
-        <v>2.39833</v>
+        <v>1.33293</v>
       </c>
       <c r="C142" s="33">
-        <v>0.66733</v>
+        <v>0.37998</v>
       </c>
       <c r="D142">
-        <v>130</v>
+        <v>85</v>
       </c>
       <c r="E142">
-        <v>100</v>
+        <v>65</v>
       </c>
     </row>
     <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>333</v>
+        <v>322</v>
       </c>
       <c r="B143" s="33">
-        <v>2.95304</v>
+        <v>1.68126</v>
       </c>
       <c r="C143" s="33">
-        <v>0.75045</v>
+        <v>0.36681</v>
       </c>
       <c r="D143">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="E143">
-        <v>120</v>
+        <v>75</v>
       </c>
     </row>
     <row r="144" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="B144" s="33">
-        <v>3.63758</v>
+        <v>2.1044</v>
       </c>
       <c r="C144" s="33">
-        <v>0.88701</v>
+        <v>0.4821</v>
       </c>
       <c r="D144">
-        <v>175</v>
+        <v>115</v>
       </c>
       <c r="E144">
-        <v>135</v>
+        <v>90</v>
       </c>
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>342</v>
+        <v>325</v>
       </c>
       <c r="B145" s="33">
-        <v>4.5658</v>
+        <v>2.39833</v>
       </c>
       <c r="C145" s="33">
-        <v>1.09956</v>
+        <v>0.66733</v>
       </c>
       <c r="D145">
-        <v>200</v>
+        <v>130</v>
       </c>
       <c r="E145">
-        <v>155</v>
+        <v>100</v>
       </c>
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>58</v>
+        <v>333</v>
       </c>
       <c r="B146" s="33">
-        <v>5.73045</v>
+        <v>2.95304</v>
       </c>
       <c r="C146" s="33">
-        <v>1.2278</v>
+        <v>0.75045</v>
       </c>
       <c r="D146">
-        <v>230</v>
+        <v>150</v>
       </c>
       <c r="E146">
-        <v>180</v>
+        <v>120</v>
       </c>
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>367</v>
+        <v>422</v>
       </c>
       <c r="B147" s="33">
-        <v>6.64016</v>
+        <v>3.63758</v>
       </c>
       <c r="C147" s="33">
-        <v>1.49616</v>
+        <v>0.88701</v>
       </c>
       <c r="D147">
-        <v>255</v>
+        <v>175</v>
       </c>
       <c r="E147">
-        <v>205</v>
+        <v>135</v>
       </c>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>351</v>
+        <v>342</v>
       </c>
       <c r="B148" s="33">
-        <v>7.9632</v>
+        <v>4.5658</v>
       </c>
       <c r="C148" s="33">
-        <v>2.06137</v>
+        <v>1.09956</v>
       </c>
       <c r="D148">
-        <v>285</v>
+        <v>200</v>
       </c>
       <c r="E148">
-        <v>230</v>
+        <v>155</v>
       </c>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B149" s="33">
-        <v>9.32416</v>
+        <v>5.73045</v>
       </c>
       <c r="C149" s="33">
-        <v>2.10412</v>
+        <v>1.2278</v>
       </c>
       <c r="D149">
-        <v>310</v>
+        <v>230</v>
       </c>
       <c r="E149">
-        <v>250</v>
+        <v>180</v>
       </c>
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
       <c r="B150" s="33">
-        <v>10.60671</v>
+        <v>6.64016</v>
       </c>
       <c r="C150" s="33">
-        <v>2.45797</v>
+        <v>1.49616</v>
       </c>
       <c r="D150">
-        <v>335</v>
+        <v>255</v>
       </c>
       <c r="E150">
-        <v>270</v>
+        <v>205</v>
       </c>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>423</v>
+        <v>351</v>
       </c>
       <c r="B151" s="33">
-        <v>11.334</v>
+        <v>7.9632</v>
       </c>
       <c r="C151" s="33">
-        <v>2.589</v>
+        <v>2.06137</v>
       </c>
       <c r="D151">
-        <v>355</v>
+        <v>285</v>
       </c>
       <c r="E151">
-        <v>290</v>
+        <v>230</v>
       </c>
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>424</v>
+        <v>60</v>
       </c>
       <c r="B152" s="33">
-        <v>13.30059</v>
+        <v>9.32416</v>
       </c>
       <c r="C152" s="33">
-        <v>2.7204</v>
+        <v>2.10412</v>
       </c>
       <c r="D152">
-        <v>380</v>
+        <v>310</v>
       </c>
       <c r="E152">
-        <v>310</v>
+        <v>250</v>
       </c>
     </row>
     <row r="153" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>55</v>
+        <v>359</v>
       </c>
       <c r="B153" s="33">
-        <v>16.57382</v>
+        <v>10.60671</v>
       </c>
       <c r="C153" s="33">
-        <v>3.44354</v>
+        <v>2.45797</v>
       </c>
       <c r="D153">
-        <v>420</v>
+        <v>335</v>
       </c>
       <c r="E153">
-        <v>340</v>
+        <v>270</v>
       </c>
     </row>
     <row r="154" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="B154" s="33">
-        <v>0</v>
+        <v>11.334</v>
       </c>
       <c r="C154" s="33">
-        <v>4.809</v>
+        <v>2.589</v>
       </c>
       <c r="D154">
-        <v>460</v>
+        <v>355</v>
       </c>
       <c r="E154">
-        <v>375</v>
+        <v>290</v>
       </c>
     </row>
     <row r="155" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="B155" s="33">
-        <v>25.921</v>
+        <v>13.30059</v>
       </c>
       <c r="C155" s="33">
-        <v>4.859</v>
+        <v>2.7204</v>
       </c>
       <c r="D155">
-        <v>475</v>
+        <v>380</v>
       </c>
       <c r="E155">
-        <v>385</v>
+        <v>310</v>
       </c>
     </row>
     <row r="156" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>427</v>
+        <v>55</v>
       </c>
       <c r="B156" s="33">
-        <v>0</v>
+        <v>16.57382</v>
       </c>
       <c r="C156" s="33">
-        <v>0</v>
+        <v>3.44354</v>
       </c>
       <c r="D156">
-        <v>490</v>
+        <v>420</v>
       </c>
       <c r="E156">
-        <v>395</v>
+        <v>340</v>
       </c>
     </row>
     <row r="157" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
       <c r="B157" s="33">
         <v>0</v>
       </c>
       <c r="C157" s="33">
-        <v>7.566</v>
+        <v>4.809</v>
       </c>
       <c r="D157">
-        <v>520</v>
+        <v>460</v>
       </c>
       <c r="E157">
-        <v>425</v>
+        <v>375</v>
       </c>
     </row>
     <row r="158" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
+        <v>426</v>
+      </c>
+      <c r="B158" s="33">
+        <v>25.921</v>
+      </c>
+      <c r="C158" s="33">
+        <v>4.859</v>
+      </c>
+      <c r="D158">
+        <v>475</v>
+      </c>
+      <c r="E158">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A159" t="s">
+        <v>427</v>
+      </c>
+      <c r="B159" s="33">
+        <v>0</v>
+      </c>
+      <c r="C159" s="33">
+        <v>0</v>
+      </c>
+      <c r="D159">
+        <v>490</v>
+      </c>
+      <c r="E159">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A160" t="s">
+        <v>428</v>
+      </c>
+      <c r="B160" s="33">
+        <v>0</v>
+      </c>
+      <c r="C160" s="33">
+        <v>7.566</v>
+      </c>
+      <c r="D160">
+        <v>520</v>
+      </c>
+      <c r="E160">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A161" t="s">
         <v>429</v>
       </c>
-      <c r="B158" s="33">
+      <c r="B161" s="33">
         <v>34.398</v>
       </c>
-      <c r="C158" s="33">
+      <c r="C161" s="33">
         <v>6.668</v>
       </c>
-      <c r="D158">
+      <c r="D161">
         <v>545</v>
       </c>
-      <c r="E158">
+      <c r="E161">
         <v>445</v>
       </c>
     </row>
-    <row r="159" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A159" s="2" t="s">
+    <row r="162" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A162" s="2" t="s">
         <v>430</v>
       </c>
     </row>
@@ -8107,10 +8128,10 @@
   </sheetData>
   <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" sqref="D10:D28">
-      <formula1>RateCard!$A$134:$A$158</formula1>
+      <formula1>RateCard!$A$137:$A$161</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="D5:D28">
-      <formula1>RateCard!$A$134:$A$158</formula1>
+      <formula1>RateCard!$A$137:$A$161</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="E10:E28">
       <formula1>"Cu,Al"</formula1>

</xml_diff>